<commit_message>
Malla con Compensatorios Obligatorios
</commit_message>
<xml_diff>
--- a/malla_historica.xlsx
+++ b/malla_historica.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E369"/>
+  <dimension ref="A1:F369"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -446,6 +446,11 @@
           <t>Noches_Acum</t>
         </is>
       </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Deuda_Compensatorio</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -467,6 +472,7 @@
         <v>46204</v>
       </c>
       <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -488,6 +494,7 @@
         <v>46204</v>
       </c>
       <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -509,6 +516,7 @@
         <v>46204</v>
       </c>
       <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -530,6 +538,7 @@
         <v>46204</v>
       </c>
       <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -551,6 +560,7 @@
         <v>46205</v>
       </c>
       <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -572,6 +582,7 @@
         <v>46205</v>
       </c>
       <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -593,6 +604,7 @@
         <v>46205</v>
       </c>
       <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -614,6 +626,7 @@
         <v>46205</v>
       </c>
       <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -635,6 +648,7 @@
         <v>46206</v>
       </c>
       <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -656,6 +670,7 @@
         <v>46206</v>
       </c>
       <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -677,6 +692,7 @@
         <v>46206</v>
       </c>
       <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -698,6 +714,7 @@
         <v>46206</v>
       </c>
       <c r="E13" t="inlineStr"/>
+      <c r="F13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -719,6 +736,7 @@
         <v>46207</v>
       </c>
       <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -740,6 +758,7 @@
         <v>46207</v>
       </c>
       <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -761,6 +780,7 @@
         <v>46207</v>
       </c>
       <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -782,6 +802,7 @@
         <v>46207</v>
       </c>
       <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -803,6 +824,7 @@
         <v>46208</v>
       </c>
       <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -824,6 +846,7 @@
         <v>46208</v>
       </c>
       <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -845,6 +868,7 @@
         <v>46208</v>
       </c>
       <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -866,6 +890,7 @@
         <v>46208</v>
       </c>
       <c r="E21" t="inlineStr"/>
+      <c r="F21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -887,6 +912,7 @@
         <v>46209</v>
       </c>
       <c r="E22" t="inlineStr"/>
+      <c r="F22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -908,6 +934,7 @@
         <v>46209</v>
       </c>
       <c r="E23" t="inlineStr"/>
+      <c r="F23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -929,6 +956,7 @@
         <v>46209</v>
       </c>
       <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -950,6 +978,7 @@
         <v>46209</v>
       </c>
       <c r="E25" t="inlineStr"/>
+      <c r="F25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -971,6 +1000,7 @@
         <v>46210</v>
       </c>
       <c r="E26" t="inlineStr"/>
+      <c r="F26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -992,6 +1022,7 @@
         <v>46210</v>
       </c>
       <c r="E27" t="inlineStr"/>
+      <c r="F27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1013,6 +1044,7 @@
         <v>46210</v>
       </c>
       <c r="E28" t="inlineStr"/>
+      <c r="F28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1034,6 +1066,7 @@
         <v>46210</v>
       </c>
       <c r="E29" t="inlineStr"/>
+      <c r="F29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1055,6 +1088,7 @@
         <v>46211</v>
       </c>
       <c r="E30" t="inlineStr"/>
+      <c r="F30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1076,6 +1110,7 @@
         <v>46211</v>
       </c>
       <c r="E31" t="inlineStr"/>
+      <c r="F31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1097,6 +1132,7 @@
         <v>46211</v>
       </c>
       <c r="E32" t="inlineStr"/>
+      <c r="F32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1118,6 +1154,7 @@
         <v>46211</v>
       </c>
       <c r="E33" t="inlineStr"/>
+      <c r="F33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1139,6 +1176,7 @@
         <v>46212</v>
       </c>
       <c r="E34" t="inlineStr"/>
+      <c r="F34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1160,6 +1198,7 @@
         <v>46212</v>
       </c>
       <c r="E35" t="inlineStr"/>
+      <c r="F35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1181,6 +1220,7 @@
         <v>46212</v>
       </c>
       <c r="E36" t="inlineStr"/>
+      <c r="F36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1202,6 +1242,7 @@
         <v>46212</v>
       </c>
       <c r="E37" t="inlineStr"/>
+      <c r="F37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1223,6 +1264,7 @@
         <v>46213</v>
       </c>
       <c r="E38" t="inlineStr"/>
+      <c r="F38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1244,6 +1286,7 @@
         <v>46213</v>
       </c>
       <c r="E39" t="inlineStr"/>
+      <c r="F39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -1265,6 +1308,7 @@
         <v>46213</v>
       </c>
       <c r="E40" t="inlineStr"/>
+      <c r="F40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -1286,6 +1330,7 @@
         <v>46213</v>
       </c>
       <c r="E41" t="inlineStr"/>
+      <c r="F41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -1307,6 +1352,7 @@
         <v>46214</v>
       </c>
       <c r="E42" t="inlineStr"/>
+      <c r="F42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -1328,6 +1374,7 @@
         <v>46214</v>
       </c>
       <c r="E43" t="inlineStr"/>
+      <c r="F43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -1349,6 +1396,7 @@
         <v>46214</v>
       </c>
       <c r="E44" t="inlineStr"/>
+      <c r="F44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -1370,6 +1418,7 @@
         <v>46214</v>
       </c>
       <c r="E45" t="inlineStr"/>
+      <c r="F45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -1391,6 +1440,7 @@
         <v>46215</v>
       </c>
       <c r="E46" t="inlineStr"/>
+      <c r="F46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -1412,6 +1462,7 @@
         <v>46215</v>
       </c>
       <c r="E47" t="inlineStr"/>
+      <c r="F47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -1433,6 +1484,7 @@
         <v>46215</v>
       </c>
       <c r="E48" t="inlineStr"/>
+      <c r="F48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -1454,6 +1506,7 @@
         <v>46215</v>
       </c>
       <c r="E49" t="inlineStr"/>
+      <c r="F49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -1475,6 +1528,7 @@
         <v>46216</v>
       </c>
       <c r="E50" t="inlineStr"/>
+      <c r="F50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -1496,6 +1550,7 @@
         <v>46216</v>
       </c>
       <c r="E51" t="inlineStr"/>
+      <c r="F51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -1517,6 +1572,7 @@
         <v>46216</v>
       </c>
       <c r="E52" t="inlineStr"/>
+      <c r="F52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -1538,6 +1594,7 @@
         <v>46216</v>
       </c>
       <c r="E53" t="inlineStr"/>
+      <c r="F53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -1559,6 +1616,7 @@
         <v>46217</v>
       </c>
       <c r="E54" t="inlineStr"/>
+      <c r="F54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -1580,6 +1638,7 @@
         <v>46217</v>
       </c>
       <c r="E55" t="inlineStr"/>
+      <c r="F55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -1601,6 +1660,7 @@
         <v>46217</v>
       </c>
       <c r="E56" t="inlineStr"/>
+      <c r="F56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -1622,6 +1682,7 @@
         <v>46217</v>
       </c>
       <c r="E57" t="inlineStr"/>
+      <c r="F57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -1643,6 +1704,7 @@
         <v>46218</v>
       </c>
       <c r="E58" t="inlineStr"/>
+      <c r="F58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -1664,6 +1726,7 @@
         <v>46218</v>
       </c>
       <c r="E59" t="inlineStr"/>
+      <c r="F59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -1685,6 +1748,7 @@
         <v>46218</v>
       </c>
       <c r="E60" t="inlineStr"/>
+      <c r="F60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -1706,6 +1770,7 @@
         <v>46218</v>
       </c>
       <c r="E61" t="inlineStr"/>
+      <c r="F61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -1727,6 +1792,7 @@
         <v>46219</v>
       </c>
       <c r="E62" t="inlineStr"/>
+      <c r="F62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -1748,6 +1814,7 @@
         <v>46219</v>
       </c>
       <c r="E63" t="inlineStr"/>
+      <c r="F63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -1769,6 +1836,7 @@
         <v>46219</v>
       </c>
       <c r="E64" t="inlineStr"/>
+      <c r="F64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -1790,6 +1858,7 @@
         <v>46219</v>
       </c>
       <c r="E65" t="inlineStr"/>
+      <c r="F65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -1811,6 +1880,7 @@
         <v>46220</v>
       </c>
       <c r="E66" t="inlineStr"/>
+      <c r="F66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -1832,6 +1902,7 @@
         <v>46220</v>
       </c>
       <c r="E67" t="inlineStr"/>
+      <c r="F67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -1853,6 +1924,7 @@
         <v>46220</v>
       </c>
       <c r="E68" t="inlineStr"/>
+      <c r="F68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -1874,6 +1946,7 @@
         <v>46220</v>
       </c>
       <c r="E69" t="inlineStr"/>
+      <c r="F69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -1895,6 +1968,7 @@
         <v>46221</v>
       </c>
       <c r="E70" t="inlineStr"/>
+      <c r="F70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -1916,6 +1990,7 @@
         <v>46221</v>
       </c>
       <c r="E71" t="inlineStr"/>
+      <c r="F71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -1937,6 +2012,7 @@
         <v>46221</v>
       </c>
       <c r="E72" t="inlineStr"/>
+      <c r="F72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -1958,6 +2034,7 @@
         <v>46221</v>
       </c>
       <c r="E73" t="inlineStr"/>
+      <c r="F73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -1979,6 +2056,7 @@
         <v>46222</v>
       </c>
       <c r="E74" t="inlineStr"/>
+      <c r="F74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -2000,6 +2078,7 @@
         <v>46222</v>
       </c>
       <c r="E75" t="inlineStr"/>
+      <c r="F75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -2021,6 +2100,7 @@
         <v>46222</v>
       </c>
       <c r="E76" t="inlineStr"/>
+      <c r="F76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -2042,6 +2122,7 @@
         <v>46222</v>
       </c>
       <c r="E77" t="inlineStr"/>
+      <c r="F77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -2063,6 +2144,7 @@
         <v>46223</v>
       </c>
       <c r="E78" t="inlineStr"/>
+      <c r="F78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -2084,6 +2166,7 @@
         <v>46223</v>
       </c>
       <c r="E79" t="inlineStr"/>
+      <c r="F79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -2105,6 +2188,7 @@
         <v>46223</v>
       </c>
       <c r="E80" t="inlineStr"/>
+      <c r="F80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -2126,6 +2210,7 @@
         <v>46223</v>
       </c>
       <c r="E81" t="inlineStr"/>
+      <c r="F81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -2147,6 +2232,7 @@
         <v>46224</v>
       </c>
       <c r="E82" t="inlineStr"/>
+      <c r="F82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -2168,6 +2254,7 @@
         <v>46224</v>
       </c>
       <c r="E83" t="inlineStr"/>
+      <c r="F83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -2189,6 +2276,7 @@
         <v>46224</v>
       </c>
       <c r="E84" t="inlineStr"/>
+      <c r="F84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -2210,6 +2298,7 @@
         <v>46224</v>
       </c>
       <c r="E85" t="inlineStr"/>
+      <c r="F85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -2231,6 +2320,7 @@
         <v>46225</v>
       </c>
       <c r="E86" t="inlineStr"/>
+      <c r="F86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -2252,6 +2342,7 @@
         <v>46225</v>
       </c>
       <c r="E87" t="inlineStr"/>
+      <c r="F87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -2273,6 +2364,7 @@
         <v>46225</v>
       </c>
       <c r="E88" t="inlineStr"/>
+      <c r="F88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -2294,6 +2386,7 @@
         <v>46225</v>
       </c>
       <c r="E89" t="inlineStr"/>
+      <c r="F89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -2315,6 +2408,7 @@
         <v>46226</v>
       </c>
       <c r="E90" t="inlineStr"/>
+      <c r="F90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -2336,6 +2430,7 @@
         <v>46226</v>
       </c>
       <c r="E91" t="inlineStr"/>
+      <c r="F91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -2357,6 +2452,7 @@
         <v>46226</v>
       </c>
       <c r="E92" t="inlineStr"/>
+      <c r="F92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -2378,6 +2474,7 @@
         <v>46226</v>
       </c>
       <c r="E93" t="inlineStr"/>
+      <c r="F93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -2399,6 +2496,7 @@
         <v>46227</v>
       </c>
       <c r="E94" t="inlineStr"/>
+      <c r="F94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -2420,6 +2518,7 @@
         <v>46227</v>
       </c>
       <c r="E95" t="inlineStr"/>
+      <c r="F95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -2441,6 +2540,7 @@
         <v>46227</v>
       </c>
       <c r="E96" t="inlineStr"/>
+      <c r="F96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -2462,6 +2562,7 @@
         <v>46227</v>
       </c>
       <c r="E97" t="inlineStr"/>
+      <c r="F97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -2483,6 +2584,7 @@
         <v>46228</v>
       </c>
       <c r="E98" t="inlineStr"/>
+      <c r="F98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -2504,6 +2606,7 @@
         <v>46228</v>
       </c>
       <c r="E99" t="inlineStr"/>
+      <c r="F99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -2525,6 +2628,7 @@
         <v>46228</v>
       </c>
       <c r="E100" t="inlineStr"/>
+      <c r="F100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -2546,6 +2650,7 @@
         <v>46228</v>
       </c>
       <c r="E101" t="inlineStr"/>
+      <c r="F101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -2567,6 +2672,7 @@
         <v>46229</v>
       </c>
       <c r="E102" t="inlineStr"/>
+      <c r="F102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -2588,6 +2694,7 @@
         <v>46229</v>
       </c>
       <c r="E103" t="inlineStr"/>
+      <c r="F103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -2609,6 +2716,7 @@
         <v>46229</v>
       </c>
       <c r="E104" t="inlineStr"/>
+      <c r="F104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -2630,6 +2738,7 @@
         <v>46229</v>
       </c>
       <c r="E105" t="inlineStr"/>
+      <c r="F105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -2651,6 +2760,7 @@
         <v>46230</v>
       </c>
       <c r="E106" t="inlineStr"/>
+      <c r="F106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -2672,6 +2782,7 @@
         <v>46230</v>
       </c>
       <c r="E107" t="inlineStr"/>
+      <c r="F107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -2693,6 +2804,7 @@
         <v>46230</v>
       </c>
       <c r="E108" t="inlineStr"/>
+      <c r="F108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -2714,6 +2826,7 @@
         <v>46230</v>
       </c>
       <c r="E109" t="inlineStr"/>
+      <c r="F109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -2735,6 +2848,7 @@
         <v>46231</v>
       </c>
       <c r="E110" t="inlineStr"/>
+      <c r="F110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -2756,6 +2870,7 @@
         <v>46231</v>
       </c>
       <c r="E111" t="inlineStr"/>
+      <c r="F111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -2777,6 +2892,7 @@
         <v>46231</v>
       </c>
       <c r="E112" t="inlineStr"/>
+      <c r="F112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -2798,6 +2914,7 @@
         <v>46231</v>
       </c>
       <c r="E113" t="inlineStr"/>
+      <c r="F113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -2819,6 +2936,7 @@
         <v>46232</v>
       </c>
       <c r="E114" t="inlineStr"/>
+      <c r="F114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -2840,6 +2958,7 @@
         <v>46232</v>
       </c>
       <c r="E115" t="inlineStr"/>
+      <c r="F115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -2861,6 +2980,7 @@
         <v>46232</v>
       </c>
       <c r="E116" t="inlineStr"/>
+      <c r="F116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -2882,6 +3002,7 @@
         <v>46232</v>
       </c>
       <c r="E117" t="inlineStr"/>
+      <c r="F117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -2903,6 +3024,7 @@
         <v>46233</v>
       </c>
       <c r="E118" t="inlineStr"/>
+      <c r="F118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -2924,6 +3046,7 @@
         <v>46233</v>
       </c>
       <c r="E119" t="inlineStr"/>
+      <c r="F119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -2945,6 +3068,7 @@
         <v>46233</v>
       </c>
       <c r="E120" t="inlineStr"/>
+      <c r="F120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -2966,6 +3090,7 @@
         <v>46233</v>
       </c>
       <c r="E121" t="inlineStr"/>
+      <c r="F121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -2987,6 +3112,7 @@
         <v>46234</v>
       </c>
       <c r="E122" t="inlineStr"/>
+      <c r="F122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -3008,6 +3134,7 @@
         <v>46234</v>
       </c>
       <c r="E123" t="inlineStr"/>
+      <c r="F123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -3029,6 +3156,7 @@
         <v>46234</v>
       </c>
       <c r="E124" t="inlineStr"/>
+      <c r="F124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -3050,6 +3178,7 @@
         <v>46234</v>
       </c>
       <c r="E125" t="inlineStr"/>
+      <c r="F125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -3073,6 +3202,7 @@
       <c r="E126" t="n">
         <v>0</v>
       </c>
+      <c r="F126" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -3096,6 +3226,7 @@
       <c r="E127" t="n">
         <v>0</v>
       </c>
+      <c r="F127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -3119,6 +3250,7 @@
       <c r="E128" t="n">
         <v>1</v>
       </c>
+      <c r="F128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -3142,6 +3274,7 @@
       <c r="E129" t="n">
         <v>0</v>
       </c>
+      <c r="F129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -3165,6 +3298,7 @@
       <c r="E130" t="n">
         <v>0</v>
       </c>
+      <c r="F130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -3188,6 +3322,7 @@
       <c r="E131" t="n">
         <v>0</v>
       </c>
+      <c r="F131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -3211,6 +3346,7 @@
       <c r="E132" t="n">
         <v>2</v>
       </c>
+      <c r="F132" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -3234,6 +3370,7 @@
       <c r="E133" t="n">
         <v>0</v>
       </c>
+      <c r="F133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -3257,6 +3394,7 @@
       <c r="E134" t="n">
         <v>1</v>
       </c>
+      <c r="F134" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -3280,6 +3418,7 @@
       <c r="E135" t="n">
         <v>0</v>
       </c>
+      <c r="F135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -3303,6 +3442,7 @@
       <c r="E136" t="n">
         <v>0</v>
       </c>
+      <c r="F136" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -3326,6 +3466,7 @@
       <c r="E137" t="n">
         <v>0</v>
       </c>
+      <c r="F137" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -3349,6 +3490,7 @@
       <c r="E138" t="n">
         <v>2</v>
       </c>
+      <c r="F138" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -3372,6 +3514,7 @@
       <c r="E139" t="n">
         <v>0</v>
       </c>
+      <c r="F139" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -3395,6 +3538,7 @@
       <c r="E140" t="n">
         <v>0</v>
       </c>
+      <c r="F140" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -3418,6 +3562,7 @@
       <c r="E141" t="n">
         <v>0</v>
       </c>
+      <c r="F141" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -3441,6 +3586,7 @@
       <c r="E142" t="n">
         <v>3</v>
       </c>
+      <c r="F142" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -3464,6 +3610,7 @@
       <c r="E143" t="n">
         <v>0</v>
       </c>
+      <c r="F143" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -3487,6 +3634,7 @@
       <c r="E144" t="n">
         <v>0</v>
       </c>
+      <c r="F144" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -3510,6 +3658,7 @@
       <c r="E145" t="n">
         <v>0</v>
       </c>
+      <c r="F145" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -3533,6 +3682,7 @@
       <c r="E146" t="n">
         <v>4</v>
       </c>
+      <c r="F146" t="inlineStr"/>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -3556,6 +3706,7 @@
       <c r="E147" t="n">
         <v>1</v>
       </c>
+      <c r="F147" t="inlineStr"/>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -3579,6 +3730,7 @@
       <c r="E148" t="n">
         <v>0</v>
       </c>
+      <c r="F148" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -3602,6 +3754,7 @@
       <c r="E149" t="n">
         <v>0</v>
       </c>
+      <c r="F149" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -3625,6 +3778,7 @@
       <c r="E150" t="n">
         <v>5</v>
       </c>
+      <c r="F150" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -3648,6 +3802,7 @@
       <c r="E151" t="n">
         <v>2</v>
       </c>
+      <c r="F151" t="inlineStr"/>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -3671,6 +3826,7 @@
       <c r="E152" t="n">
         <v>0</v>
       </c>
+      <c r="F152" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -3694,6 +3850,7 @@
       <c r="E153" t="n">
         <v>0</v>
       </c>
+      <c r="F153" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -3717,6 +3874,7 @@
       <c r="E154" t="n">
         <v>6</v>
       </c>
+      <c r="F154" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -3740,6 +3898,7 @@
       <c r="E155" t="n">
         <v>3</v>
       </c>
+      <c r="F155" t="inlineStr"/>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -3763,6 +3922,7 @@
       <c r="E156" t="n">
         <v>0</v>
       </c>
+      <c r="F156" t="inlineStr"/>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
@@ -3786,6 +3946,7 @@
       <c r="E157" t="n">
         <v>0</v>
       </c>
+      <c r="F157" t="inlineStr"/>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
@@ -3809,6 +3970,7 @@
       <c r="E158" t="n">
         <v>7</v>
       </c>
+      <c r="F158" t="inlineStr"/>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -3832,6 +3994,7 @@
       <c r="E159" t="n">
         <v>0</v>
       </c>
+      <c r="F159" t="inlineStr"/>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -3855,6 +4018,7 @@
       <c r="E160" t="n">
         <v>0</v>
       </c>
+      <c r="F160" t="inlineStr"/>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
@@ -3878,6 +4042,7 @@
       <c r="E161" t="n">
         <v>0</v>
       </c>
+      <c r="F161" t="inlineStr"/>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
@@ -3901,6 +4066,7 @@
       <c r="E162" t="n">
         <v>0</v>
       </c>
+      <c r="F162" t="inlineStr"/>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
@@ -3924,6 +4090,7 @@
       <c r="E163" t="n">
         <v>1</v>
       </c>
+      <c r="F163" t="inlineStr"/>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
@@ -3947,6 +4114,7 @@
       <c r="E164" t="n">
         <v>0</v>
       </c>
+      <c r="F164" t="inlineStr"/>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
@@ -3970,6 +4138,7 @@
       <c r="E165" t="n">
         <v>0</v>
       </c>
+      <c r="F165" t="inlineStr"/>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
@@ -3993,6 +4162,7 @@
       <c r="E166" t="n">
         <v>0</v>
       </c>
+      <c r="F166" t="inlineStr"/>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
@@ -4016,6 +4186,7 @@
       <c r="E167" t="n">
         <v>2</v>
       </c>
+      <c r="F167" t="inlineStr"/>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
@@ -4039,6 +4210,7 @@
       <c r="E168" t="n">
         <v>0</v>
       </c>
+      <c r="F168" t="inlineStr"/>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
@@ -4062,6 +4234,7 @@
       <c r="E169" t="n">
         <v>0</v>
       </c>
+      <c r="F169" t="inlineStr"/>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
@@ -4085,6 +4258,7 @@
       <c r="E170" t="n">
         <v>0</v>
       </c>
+      <c r="F170" t="inlineStr"/>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
@@ -4108,6 +4282,7 @@
       <c r="E171" t="n">
         <v>3</v>
       </c>
+      <c r="F171" t="inlineStr"/>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
@@ -4131,6 +4306,7 @@
       <c r="E172" t="n">
         <v>0</v>
       </c>
+      <c r="F172" t="inlineStr"/>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
@@ -4154,6 +4330,7 @@
       <c r="E173" t="n">
         <v>0</v>
       </c>
+      <c r="F173" t="inlineStr"/>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
@@ -4177,6 +4354,7 @@
       <c r="E174" t="n">
         <v>0</v>
       </c>
+      <c r="F174" t="inlineStr"/>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
@@ -4200,6 +4378,7 @@
       <c r="E175" t="n">
         <v>4</v>
       </c>
+      <c r="F175" t="inlineStr"/>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
@@ -4223,6 +4402,7 @@
       <c r="E176" t="n">
         <v>0</v>
       </c>
+      <c r="F176" t="inlineStr"/>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
@@ -4246,6 +4426,7 @@
       <c r="E177" t="n">
         <v>1</v>
       </c>
+      <c r="F177" t="inlineStr"/>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
@@ -4269,6 +4450,7 @@
       <c r="E178" t="n">
         <v>0</v>
       </c>
+      <c r="F178" t="inlineStr"/>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
@@ -4292,6 +4474,7 @@
       <c r="E179" t="n">
         <v>5</v>
       </c>
+      <c r="F179" t="inlineStr"/>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
@@ -4315,6 +4498,7 @@
       <c r="E180" t="n">
         <v>0</v>
       </c>
+      <c r="F180" t="inlineStr"/>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
@@ -4338,6 +4522,7 @@
       <c r="E181" t="n">
         <v>2</v>
       </c>
+      <c r="F181" t="inlineStr"/>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
@@ -4361,6 +4546,7 @@
       <c r="E182" t="n">
         <v>0</v>
       </c>
+      <c r="F182" t="inlineStr"/>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
@@ -4384,6 +4570,7 @@
       <c r="E183" t="n">
         <v>6</v>
       </c>
+      <c r="F183" t="inlineStr"/>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
@@ -4407,6 +4594,7 @@
       <c r="E184" t="n">
         <v>0</v>
       </c>
+      <c r="F184" t="inlineStr"/>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
@@ -4430,6 +4618,7 @@
       <c r="E185" t="n">
         <v>3</v>
       </c>
+      <c r="F185" t="inlineStr"/>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
@@ -4453,6 +4642,7 @@
       <c r="E186" t="n">
         <v>0</v>
       </c>
+      <c r="F186" t="inlineStr"/>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
@@ -4476,6 +4666,7 @@
       <c r="E187" t="n">
         <v>7</v>
       </c>
+      <c r="F187" t="inlineStr"/>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
@@ -4499,6 +4690,7 @@
       <c r="E188" t="n">
         <v>0</v>
       </c>
+      <c r="F188" t="inlineStr"/>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
@@ -4522,6 +4714,7 @@
       <c r="E189" t="n">
         <v>4</v>
       </c>
+      <c r="F189" t="inlineStr"/>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
@@ -4545,6 +4738,7 @@
       <c r="E190" t="n">
         <v>0</v>
       </c>
+      <c r="F190" t="inlineStr"/>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
@@ -4568,6 +4762,7 @@
       <c r="E191" t="n">
         <v>0</v>
       </c>
+      <c r="F191" t="inlineStr"/>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
@@ -4591,6 +4786,7 @@
       <c r="E192" t="n">
         <v>0</v>
       </c>
+      <c r="F192" t="inlineStr"/>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
@@ -4614,6 +4810,7 @@
       <c r="E193" t="n">
         <v>5</v>
       </c>
+      <c r="F193" t="inlineStr"/>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
@@ -4637,6 +4834,7 @@
       <c r="E194" t="n">
         <v>0</v>
       </c>
+      <c r="F194" t="inlineStr"/>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
@@ -4660,6 +4858,7 @@
       <c r="E195" t="n">
         <v>0</v>
       </c>
+      <c r="F195" t="inlineStr"/>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
@@ -4683,6 +4882,7 @@
       <c r="E196" t="n">
         <v>0</v>
       </c>
+      <c r="F196" t="inlineStr"/>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
@@ -4706,6 +4906,7 @@
       <c r="E197" t="n">
         <v>6</v>
       </c>
+      <c r="F197" t="inlineStr"/>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
@@ -4729,6 +4930,7 @@
       <c r="E198" t="n">
         <v>0</v>
       </c>
+      <c r="F198" t="inlineStr"/>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
@@ -4752,6 +4954,7 @@
       <c r="E199" t="n">
         <v>0</v>
       </c>
+      <c r="F199" t="inlineStr"/>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
@@ -4775,6 +4978,7 @@
       <c r="E200" t="n">
         <v>1</v>
       </c>
+      <c r="F200" t="inlineStr"/>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
@@ -4798,6 +5002,7 @@
       <c r="E201" t="n">
         <v>7</v>
       </c>
+      <c r="F201" t="inlineStr"/>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
@@ -4821,6 +5026,7 @@
       <c r="E202" t="n">
         <v>0</v>
       </c>
+      <c r="F202" t="inlineStr"/>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
@@ -4844,6 +5050,7 @@
       <c r="E203" t="n">
         <v>0</v>
       </c>
+      <c r="F203" t="inlineStr"/>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
@@ -4867,6 +5074,7 @@
       <c r="E204" t="n">
         <v>2</v>
       </c>
+      <c r="F204" t="inlineStr"/>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
@@ -4890,6 +5098,7 @@
       <c r="E205" t="n">
         <v>0</v>
       </c>
+      <c r="F205" t="inlineStr"/>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
@@ -4913,6 +5122,7 @@
       <c r="E206" t="n">
         <v>0</v>
       </c>
+      <c r="F206" t="inlineStr"/>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
@@ -4936,6 +5146,7 @@
       <c r="E207" t="n">
         <v>0</v>
       </c>
+      <c r="F207" t="inlineStr"/>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
@@ -4959,6 +5170,7 @@
       <c r="E208" t="n">
         <v>3</v>
       </c>
+      <c r="F208" t="inlineStr"/>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
@@ -4982,6 +5194,7 @@
       <c r="E209" t="n">
         <v>0</v>
       </c>
+      <c r="F209" t="inlineStr"/>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
@@ -5005,6 +5218,7 @@
       <c r="E210" t="n">
         <v>0</v>
       </c>
+      <c r="F210" t="inlineStr"/>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
@@ -5028,6 +5242,7 @@
       <c r="E211" t="n">
         <v>0</v>
       </c>
+      <c r="F211" t="inlineStr"/>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
@@ -5051,6 +5266,7 @@
       <c r="E212" t="n">
         <v>4</v>
       </c>
+      <c r="F212" t="inlineStr"/>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
@@ -5074,6 +5290,7 @@
       <c r="E213" t="n">
         <v>0</v>
       </c>
+      <c r="F213" t="inlineStr"/>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
@@ -5097,6 +5314,7 @@
       <c r="E214" t="n">
         <v>0</v>
       </c>
+      <c r="F214" t="inlineStr"/>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
@@ -5120,6 +5338,7 @@
       <c r="E215" t="n">
         <v>0</v>
       </c>
+      <c r="F215" t="inlineStr"/>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
@@ -5143,6 +5362,7 @@
       <c r="E216" t="n">
         <v>5</v>
       </c>
+      <c r="F216" t="inlineStr"/>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
@@ -5166,6 +5386,7 @@
       <c r="E217" t="n">
         <v>0</v>
       </c>
+      <c r="F217" t="inlineStr"/>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
@@ -5189,6 +5410,7 @@
       <c r="E218" t="n">
         <v>0</v>
       </c>
+      <c r="F218" t="inlineStr"/>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
@@ -5212,6 +5434,7 @@
       <c r="E219" t="n">
         <v>0</v>
       </c>
+      <c r="F219" t="inlineStr"/>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
@@ -5235,6 +5458,7 @@
       <c r="E220" t="n">
         <v>6</v>
       </c>
+      <c r="F220" t="inlineStr"/>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
@@ -5258,6 +5482,7 @@
       <c r="E221" t="n">
         <v>0</v>
       </c>
+      <c r="F221" t="inlineStr"/>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
@@ -5281,6 +5506,7 @@
       <c r="E222" t="n">
         <v>0</v>
       </c>
+      <c r="F222" t="inlineStr"/>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
@@ -5304,6 +5530,7 @@
       <c r="E223" t="n">
         <v>0</v>
       </c>
+      <c r="F223" t="inlineStr"/>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
@@ -5327,6 +5554,7 @@
       <c r="E224" t="n">
         <v>7</v>
       </c>
+      <c r="F224" t="inlineStr"/>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
@@ -5350,6 +5578,7 @@
       <c r="E225" t="n">
         <v>0</v>
       </c>
+      <c r="F225" t="inlineStr"/>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
@@ -5373,6 +5602,7 @@
       <c r="E226" t="n">
         <v>0</v>
       </c>
+      <c r="F226" t="inlineStr"/>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
@@ -5396,6 +5626,7 @@
       <c r="E227" t="n">
         <v>1</v>
       </c>
+      <c r="F227" t="inlineStr"/>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
@@ -5419,6 +5650,7 @@
       <c r="E228" t="n">
         <v>0</v>
       </c>
+      <c r="F228" t="inlineStr"/>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
@@ -5442,6 +5674,7 @@
       <c r="E229" t="n">
         <v>0</v>
       </c>
+      <c r="F229" t="inlineStr"/>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
@@ -5465,6 +5698,7 @@
       <c r="E230" t="n">
         <v>0</v>
       </c>
+      <c r="F230" t="inlineStr"/>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
@@ -5488,6 +5722,7 @@
       <c r="E231" t="n">
         <v>2</v>
       </c>
+      <c r="F231" t="inlineStr"/>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
@@ -5511,6 +5746,7 @@
       <c r="E232" t="n">
         <v>0</v>
       </c>
+      <c r="F232" t="inlineStr"/>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
@@ -5534,6 +5770,7 @@
       <c r="E233" t="n">
         <v>0</v>
       </c>
+      <c r="F233" t="inlineStr"/>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
@@ -5557,6 +5794,7 @@
       <c r="E234" t="n">
         <v>0</v>
       </c>
+      <c r="F234" t="inlineStr"/>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
@@ -5580,6 +5818,7 @@
       <c r="E235" t="n">
         <v>3</v>
       </c>
+      <c r="F235" t="inlineStr"/>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
@@ -5603,6 +5842,7 @@
       <c r="E236" t="n">
         <v>0</v>
       </c>
+      <c r="F236" t="inlineStr"/>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
@@ -5626,6 +5866,7 @@
       <c r="E237" t="n">
         <v>0</v>
       </c>
+      <c r="F237" t="inlineStr"/>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
@@ -5649,6 +5890,7 @@
       <c r="E238" t="n">
         <v>0</v>
       </c>
+      <c r="F238" t="inlineStr"/>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
@@ -5672,6 +5914,7 @@
       <c r="E239" t="n">
         <v>4</v>
       </c>
+      <c r="F239" t="inlineStr"/>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
@@ -5695,6 +5938,7 @@
       <c r="E240" t="n">
         <v>0</v>
       </c>
+      <c r="F240" t="inlineStr"/>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
@@ -5718,6 +5962,7 @@
       <c r="E241" t="n">
         <v>0</v>
       </c>
+      <c r="F241" t="inlineStr"/>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
@@ -5741,6 +5986,7 @@
       <c r="E242" t="n">
         <v>0</v>
       </c>
+      <c r="F242" t="inlineStr"/>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
@@ -5764,6 +6010,7 @@
       <c r="E243" t="n">
         <v>5</v>
       </c>
+      <c r="F243" t="inlineStr"/>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
@@ -5787,6 +6034,7 @@
       <c r="E244" t="n">
         <v>0</v>
       </c>
+      <c r="F244" t="inlineStr"/>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
@@ -5810,6 +6058,7 @@
       <c r="E245" t="n">
         <v>0</v>
       </c>
+      <c r="F245" t="inlineStr"/>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
@@ -5833,6 +6082,7 @@
       <c r="E246" t="n">
         <v>0</v>
       </c>
+      <c r="F246" t="inlineStr"/>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
@@ -5856,6 +6106,7 @@
       <c r="E247" t="n">
         <v>6</v>
       </c>
+      <c r="F247" t="inlineStr"/>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
@@ -5879,6 +6130,7 @@
       <c r="E248" t="n">
         <v>0</v>
       </c>
+      <c r="F248" t="inlineStr"/>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
@@ -5902,6 +6154,7 @@
       <c r="E249" t="n">
         <v>0</v>
       </c>
+      <c r="F249" t="inlineStr"/>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
@@ -5916,13 +6169,18 @@
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="D250" s="1" t="n">
         <v>46174</v>
       </c>
-      <c r="E250" t="inlineStr"/>
+      <c r="E250" t="n">
+        <v>0</v>
+      </c>
+      <c r="F250" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
@@ -5943,7 +6201,12 @@
       <c r="D251" s="1" t="n">
         <v>46174</v>
       </c>
-      <c r="E251" t="inlineStr"/>
+      <c r="E251" t="n">
+        <v>0</v>
+      </c>
+      <c r="F251" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
@@ -5964,7 +6227,12 @@
       <c r="D252" s="1" t="n">
         <v>46174</v>
       </c>
-      <c r="E252" t="inlineStr"/>
+      <c r="E252" t="n">
+        <v>0</v>
+      </c>
+      <c r="F252" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="253">
       <c r="A253" t="inlineStr">
@@ -5979,13 +6247,18 @@
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>T2</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="D253" s="1" t="n">
         <v>46174</v>
       </c>
-      <c r="E253" t="inlineStr"/>
+      <c r="E253" t="n">
+        <v>1</v>
+      </c>
+      <c r="F253" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="254">
       <c r="A254" t="inlineStr">
@@ -6000,13 +6273,18 @@
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="D254" s="1" t="n">
         <v>46175</v>
       </c>
-      <c r="E254" t="inlineStr"/>
+      <c r="E254" t="n">
+        <v>0</v>
+      </c>
+      <c r="F254" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="255">
       <c r="A255" t="inlineStr">
@@ -6027,7 +6305,12 @@
       <c r="D255" s="1" t="n">
         <v>46175</v>
       </c>
-      <c r="E255" t="inlineStr"/>
+      <c r="E255" t="n">
+        <v>0</v>
+      </c>
+      <c r="F255" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="256">
       <c r="A256" t="inlineStr">
@@ -6048,7 +6331,12 @@
       <c r="D256" s="1" t="n">
         <v>46175</v>
       </c>
-      <c r="E256" t="inlineStr"/>
+      <c r="E256" t="n">
+        <v>0</v>
+      </c>
+      <c r="F256" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="257">
       <c r="A257" t="inlineStr">
@@ -6063,13 +6351,18 @@
       </c>
       <c r="C257" t="inlineStr">
         <is>
-          <t>T2</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="D257" s="1" t="n">
         <v>46175</v>
       </c>
-      <c r="E257" t="inlineStr"/>
+      <c r="E257" t="n">
+        <v>2</v>
+      </c>
+      <c r="F257" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
@@ -6084,13 +6377,18 @@
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="D258" s="1" t="n">
         <v>46176</v>
       </c>
-      <c r="E258" t="inlineStr"/>
+      <c r="E258" t="n">
+        <v>0</v>
+      </c>
+      <c r="F258" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
@@ -6111,7 +6409,12 @@
       <c r="D259" s="1" t="n">
         <v>46176</v>
       </c>
-      <c r="E259" t="inlineStr"/>
+      <c r="E259" t="n">
+        <v>0</v>
+      </c>
+      <c r="F259" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="260">
       <c r="A260" t="inlineStr">
@@ -6132,7 +6435,12 @@
       <c r="D260" s="1" t="n">
         <v>46176</v>
       </c>
-      <c r="E260" t="inlineStr"/>
+      <c r="E260" t="n">
+        <v>0</v>
+      </c>
+      <c r="F260" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
@@ -6147,13 +6455,18 @@
       </c>
       <c r="C261" t="inlineStr">
         <is>
-          <t>T2</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="D261" s="1" t="n">
         <v>46176</v>
       </c>
-      <c r="E261" t="inlineStr"/>
+      <c r="E261" t="n">
+        <v>3</v>
+      </c>
+      <c r="F261" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
@@ -6168,13 +6481,18 @@
       </c>
       <c r="C262" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="D262" s="1" t="n">
         <v>46177</v>
       </c>
-      <c r="E262" t="inlineStr"/>
+      <c r="E262" t="n">
+        <v>0</v>
+      </c>
+      <c r="F262" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
@@ -6195,7 +6513,12 @@
       <c r="D263" s="1" t="n">
         <v>46177</v>
       </c>
-      <c r="E263" t="inlineStr"/>
+      <c r="E263" t="n">
+        <v>0</v>
+      </c>
+      <c r="F263" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="264">
       <c r="A264" t="inlineStr">
@@ -6216,7 +6539,12 @@
       <c r="D264" s="1" t="n">
         <v>46177</v>
       </c>
-      <c r="E264" t="inlineStr"/>
+      <c r="E264" t="n">
+        <v>0</v>
+      </c>
+      <c r="F264" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="265">
       <c r="A265" t="inlineStr">
@@ -6231,13 +6559,18 @@
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>T2</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="D265" s="1" t="n">
         <v>46177</v>
       </c>
-      <c r="E265" t="inlineStr"/>
+      <c r="E265" t="n">
+        <v>4</v>
+      </c>
+      <c r="F265" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="266">
       <c r="A266" t="inlineStr">
@@ -6252,13 +6585,18 @@
       </c>
       <c r="C266" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="D266" s="1" t="n">
         <v>46178</v>
       </c>
-      <c r="E266" t="inlineStr"/>
+      <c r="E266" t="n">
+        <v>0</v>
+      </c>
+      <c r="F266" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="267">
       <c r="A267" t="inlineStr">
@@ -6279,7 +6617,12 @@
       <c r="D267" s="1" t="n">
         <v>46178</v>
       </c>
-      <c r="E267" t="inlineStr"/>
+      <c r="E267" t="n">
+        <v>0</v>
+      </c>
+      <c r="F267" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="268">
       <c r="A268" t="inlineStr">
@@ -6300,7 +6643,12 @@
       <c r="D268" s="1" t="n">
         <v>46178</v>
       </c>
-      <c r="E268" t="inlineStr"/>
+      <c r="E268" t="n">
+        <v>0</v>
+      </c>
+      <c r="F268" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="269">
       <c r="A269" t="inlineStr">
@@ -6315,13 +6663,18 @@
       </c>
       <c r="C269" t="inlineStr">
         <is>
-          <t>T2</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="D269" s="1" t="n">
         <v>46178</v>
       </c>
-      <c r="E269" t="inlineStr"/>
+      <c r="E269" t="n">
+        <v>5</v>
+      </c>
+      <c r="F269" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="270">
       <c r="A270" t="inlineStr">
@@ -6336,13 +6689,18 @@
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="D270" s="1" t="n">
         <v>46179</v>
       </c>
-      <c r="E270" t="inlineStr"/>
+      <c r="E270" t="n">
+        <v>0</v>
+      </c>
+      <c r="F270" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="271">
       <c r="A271" t="inlineStr">
@@ -6363,7 +6721,12 @@
       <c r="D271" s="1" t="n">
         <v>46179</v>
       </c>
-      <c r="E271" t="inlineStr"/>
+      <c r="E271" t="n">
+        <v>0</v>
+      </c>
+      <c r="F271" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="272">
       <c r="A272" t="inlineStr">
@@ -6378,13 +6741,18 @@
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="D272" s="1" t="n">
         <v>46179</v>
       </c>
-      <c r="E272" t="inlineStr"/>
+      <c r="E272" t="n">
+        <v>0</v>
+      </c>
+      <c r="F272" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="273">
       <c r="A273" t="inlineStr">
@@ -6399,13 +6767,18 @@
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>T2</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="D273" s="1" t="n">
         <v>46179</v>
       </c>
-      <c r="E273" t="inlineStr"/>
+      <c r="E273" t="n">
+        <v>6</v>
+      </c>
+      <c r="F273" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="274">
       <c r="A274" t="inlineStr">
@@ -6426,7 +6799,12 @@
       <c r="D274" s="1" t="n">
         <v>46180</v>
       </c>
-      <c r="E274" t="inlineStr"/>
+      <c r="E274" t="n">
+        <v>1</v>
+      </c>
+      <c r="F274" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="275">
       <c r="A275" t="inlineStr">
@@ -6447,7 +6825,12 @@
       <c r="D275" s="1" t="n">
         <v>46180</v>
       </c>
-      <c r="E275" t="inlineStr"/>
+      <c r="E275" t="n">
+        <v>0</v>
+      </c>
+      <c r="F275" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="276">
       <c r="A276" t="inlineStr">
@@ -6468,7 +6851,12 @@
       <c r="D276" s="1" t="n">
         <v>46180</v>
       </c>
-      <c r="E276" t="inlineStr"/>
+      <c r="E276" t="n">
+        <v>0</v>
+      </c>
+      <c r="F276" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="277">
       <c r="A277" t="inlineStr">
@@ -6489,7 +6877,12 @@
       <c r="D277" s="1" t="n">
         <v>46180</v>
       </c>
-      <c r="E277" t="inlineStr"/>
+      <c r="E277" t="n">
+        <v>0</v>
+      </c>
+      <c r="F277" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="278">
       <c r="A278" t="inlineStr">
@@ -6510,7 +6903,12 @@
       <c r="D278" s="1" t="n">
         <v>46181</v>
       </c>
-      <c r="E278" t="inlineStr"/>
+      <c r="E278" t="n">
+        <v>2</v>
+      </c>
+      <c r="F278" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="279">
       <c r="A279" t="inlineStr">
@@ -6531,7 +6929,12 @@
       <c r="D279" s="1" t="n">
         <v>46181</v>
       </c>
-      <c r="E279" t="inlineStr"/>
+      <c r="E279" t="n">
+        <v>0</v>
+      </c>
+      <c r="F279" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="280">
       <c r="A280" t="inlineStr">
@@ -6552,7 +6955,12 @@
       <c r="D280" s="1" t="n">
         <v>46181</v>
       </c>
-      <c r="E280" t="inlineStr"/>
+      <c r="E280" t="n">
+        <v>0</v>
+      </c>
+      <c r="F280" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="281">
       <c r="A281" t="inlineStr">
@@ -6573,7 +6981,12 @@
       <c r="D281" s="1" t="n">
         <v>46181</v>
       </c>
-      <c r="E281" t="inlineStr"/>
+      <c r="E281" t="n">
+        <v>0</v>
+      </c>
+      <c r="F281" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="282">
       <c r="A282" t="inlineStr">
@@ -6594,7 +7007,12 @@
       <c r="D282" s="1" t="n">
         <v>46182</v>
       </c>
-      <c r="E282" t="inlineStr"/>
+      <c r="E282" t="n">
+        <v>3</v>
+      </c>
+      <c r="F282" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="283">
       <c r="A283" t="inlineStr">
@@ -6615,7 +7033,12 @@
       <c r="D283" s="1" t="n">
         <v>46182</v>
       </c>
-      <c r="E283" t="inlineStr"/>
+      <c r="E283" t="n">
+        <v>0</v>
+      </c>
+      <c r="F283" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="284">
       <c r="A284" t="inlineStr">
@@ -6636,7 +7059,12 @@
       <c r="D284" s="1" t="n">
         <v>46182</v>
       </c>
-      <c r="E284" t="inlineStr"/>
+      <c r="E284" t="n">
+        <v>0</v>
+      </c>
+      <c r="F284" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="285">
       <c r="A285" t="inlineStr">
@@ -6657,7 +7085,12 @@
       <c r="D285" s="1" t="n">
         <v>46182</v>
       </c>
-      <c r="E285" t="inlineStr"/>
+      <c r="E285" t="n">
+        <v>0</v>
+      </c>
+      <c r="F285" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="286">
       <c r="A286" t="inlineStr">
@@ -6678,7 +7111,12 @@
       <c r="D286" s="1" t="n">
         <v>46183</v>
       </c>
-      <c r="E286" t="inlineStr"/>
+      <c r="E286" t="n">
+        <v>4</v>
+      </c>
+      <c r="F286" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="287">
       <c r="A287" t="inlineStr">
@@ -6699,7 +7137,12 @@
       <c r="D287" s="1" t="n">
         <v>46183</v>
       </c>
-      <c r="E287" t="inlineStr"/>
+      <c r="E287" t="n">
+        <v>0</v>
+      </c>
+      <c r="F287" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="288">
       <c r="A288" t="inlineStr">
@@ -6720,7 +7163,12 @@
       <c r="D288" s="1" t="n">
         <v>46183</v>
       </c>
-      <c r="E288" t="inlineStr"/>
+      <c r="E288" t="n">
+        <v>0</v>
+      </c>
+      <c r="F288" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="289">
       <c r="A289" t="inlineStr">
@@ -6741,7 +7189,12 @@
       <c r="D289" s="1" t="n">
         <v>46183</v>
       </c>
-      <c r="E289" t="inlineStr"/>
+      <c r="E289" t="n">
+        <v>0</v>
+      </c>
+      <c r="F289" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="290">
       <c r="A290" t="inlineStr">
@@ -6762,7 +7215,12 @@
       <c r="D290" s="1" t="n">
         <v>46184</v>
       </c>
-      <c r="E290" t="inlineStr"/>
+      <c r="E290" t="n">
+        <v>5</v>
+      </c>
+      <c r="F290" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="291">
       <c r="A291" t="inlineStr">
@@ -6783,7 +7241,12 @@
       <c r="D291" s="1" t="n">
         <v>46184</v>
       </c>
-      <c r="E291" t="inlineStr"/>
+      <c r="E291" t="n">
+        <v>0</v>
+      </c>
+      <c r="F291" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="292">
       <c r="A292" t="inlineStr">
@@ -6804,7 +7267,12 @@
       <c r="D292" s="1" t="n">
         <v>46184</v>
       </c>
-      <c r="E292" t="inlineStr"/>
+      <c r="E292" t="n">
+        <v>0</v>
+      </c>
+      <c r="F292" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="293">
       <c r="A293" t="inlineStr">
@@ -6825,7 +7293,12 @@
       <c r="D293" s="1" t="n">
         <v>46184</v>
       </c>
-      <c r="E293" t="inlineStr"/>
+      <c r="E293" t="n">
+        <v>0</v>
+      </c>
+      <c r="F293" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="294">
       <c r="A294" t="inlineStr">
@@ -6846,7 +7319,12 @@
       <c r="D294" s="1" t="n">
         <v>46185</v>
       </c>
-      <c r="E294" t="inlineStr"/>
+      <c r="E294" t="n">
+        <v>6</v>
+      </c>
+      <c r="F294" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="295">
       <c r="A295" t="inlineStr">
@@ -6867,7 +7345,12 @@
       <c r="D295" s="1" t="n">
         <v>46185</v>
       </c>
-      <c r="E295" t="inlineStr"/>
+      <c r="E295" t="n">
+        <v>0</v>
+      </c>
+      <c r="F295" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="296">
       <c r="A296" t="inlineStr">
@@ -6888,7 +7371,12 @@
       <c r="D296" s="1" t="n">
         <v>46185</v>
       </c>
-      <c r="E296" t="inlineStr"/>
+      <c r="E296" t="n">
+        <v>0</v>
+      </c>
+      <c r="F296" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="297">
       <c r="A297" t="inlineStr">
@@ -6909,7 +7397,12 @@
       <c r="D297" s="1" t="n">
         <v>46185</v>
       </c>
-      <c r="E297" t="inlineStr"/>
+      <c r="E297" t="n">
+        <v>0</v>
+      </c>
+      <c r="F297" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="298">
       <c r="A298" t="inlineStr">
@@ -6930,7 +7423,12 @@
       <c r="D298" s="1" t="n">
         <v>46186</v>
       </c>
-      <c r="E298" t="inlineStr"/>
+      <c r="E298" t="n">
+        <v>0</v>
+      </c>
+      <c r="F298" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="299">
       <c r="A299" t="inlineStr">
@@ -6951,7 +7449,12 @@
       <c r="D299" s="1" t="n">
         <v>46186</v>
       </c>
-      <c r="E299" t="inlineStr"/>
+      <c r="E299" t="n">
+        <v>0</v>
+      </c>
+      <c r="F299" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="300">
       <c r="A300" t="inlineStr">
@@ -6972,7 +7475,12 @@
       <c r="D300" s="1" t="n">
         <v>46186</v>
       </c>
-      <c r="E300" t="inlineStr"/>
+      <c r="E300" t="n">
+        <v>1</v>
+      </c>
+      <c r="F300" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="301">
       <c r="A301" t="inlineStr">
@@ -6993,7 +7501,12 @@
       <c r="D301" s="1" t="n">
         <v>46186</v>
       </c>
-      <c r="E301" t="inlineStr"/>
+      <c r="E301" t="n">
+        <v>0</v>
+      </c>
+      <c r="F301" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="302">
       <c r="A302" t="inlineStr">
@@ -7014,7 +7527,12 @@
       <c r="D302" s="1" t="n">
         <v>46187</v>
       </c>
-      <c r="E302" t="inlineStr"/>
+      <c r="E302" t="n">
+        <v>1</v>
+      </c>
+      <c r="F302" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="303">
       <c r="A303" t="inlineStr">
@@ -7035,7 +7553,12 @@
       <c r="D303" s="1" t="n">
         <v>46187</v>
       </c>
-      <c r="E303" t="inlineStr"/>
+      <c r="E303" t="n">
+        <v>0</v>
+      </c>
+      <c r="F303" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="304">
       <c r="A304" t="inlineStr">
@@ -7056,7 +7579,12 @@
       <c r="D304" s="1" t="n">
         <v>46187</v>
       </c>
-      <c r="E304" t="inlineStr"/>
+      <c r="E304" t="n">
+        <v>0</v>
+      </c>
+      <c r="F304" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="305">
       <c r="A305" t="inlineStr">
@@ -7077,7 +7605,12 @@
       <c r="D305" s="1" t="n">
         <v>46187</v>
       </c>
-      <c r="E305" t="inlineStr"/>
+      <c r="E305" t="n">
+        <v>0</v>
+      </c>
+      <c r="F305" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="306">
       <c r="A306" t="inlineStr">
@@ -7098,7 +7631,12 @@
       <c r="D306" s="1" t="n">
         <v>46188</v>
       </c>
-      <c r="E306" t="inlineStr"/>
+      <c r="E306" t="n">
+        <v>2</v>
+      </c>
+      <c r="F306" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="307">
       <c r="A307" t="inlineStr">
@@ -7119,7 +7657,12 @@
       <c r="D307" s="1" t="n">
         <v>46188</v>
       </c>
-      <c r="E307" t="inlineStr"/>
+      <c r="E307" t="n">
+        <v>0</v>
+      </c>
+      <c r="F307" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="308">
       <c r="A308" t="inlineStr">
@@ -7140,7 +7683,12 @@
       <c r="D308" s="1" t="n">
         <v>46188</v>
       </c>
-      <c r="E308" t="inlineStr"/>
+      <c r="E308" t="n">
+        <v>0</v>
+      </c>
+      <c r="F308" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="309">
       <c r="A309" t="inlineStr">
@@ -7161,7 +7709,12 @@
       <c r="D309" s="1" t="n">
         <v>46188</v>
       </c>
-      <c r="E309" t="inlineStr"/>
+      <c r="E309" t="n">
+        <v>0</v>
+      </c>
+      <c r="F309" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="310">
       <c r="A310" t="inlineStr">
@@ -7182,7 +7735,12 @@
       <c r="D310" s="1" t="n">
         <v>46189</v>
       </c>
-      <c r="E310" t="inlineStr"/>
+      <c r="E310" t="n">
+        <v>3</v>
+      </c>
+      <c r="F310" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="311">
       <c r="A311" t="inlineStr">
@@ -7203,7 +7761,12 @@
       <c r="D311" s="1" t="n">
         <v>46189</v>
       </c>
-      <c r="E311" t="inlineStr"/>
+      <c r="E311" t="n">
+        <v>0</v>
+      </c>
+      <c r="F311" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="312">
       <c r="A312" t="inlineStr">
@@ -7224,7 +7787,12 @@
       <c r="D312" s="1" t="n">
         <v>46189</v>
       </c>
-      <c r="E312" t="inlineStr"/>
+      <c r="E312" t="n">
+        <v>0</v>
+      </c>
+      <c r="F312" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="313">
       <c r="A313" t="inlineStr">
@@ -7245,7 +7813,12 @@
       <c r="D313" s="1" t="n">
         <v>46189</v>
       </c>
-      <c r="E313" t="inlineStr"/>
+      <c r="E313" t="n">
+        <v>0</v>
+      </c>
+      <c r="F313" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="314">
       <c r="A314" t="inlineStr">
@@ -7266,7 +7839,12 @@
       <c r="D314" s="1" t="n">
         <v>46190</v>
       </c>
-      <c r="E314" t="inlineStr"/>
+      <c r="E314" t="n">
+        <v>4</v>
+      </c>
+      <c r="F314" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="315">
       <c r="A315" t="inlineStr">
@@ -7287,7 +7865,12 @@
       <c r="D315" s="1" t="n">
         <v>46190</v>
       </c>
-      <c r="E315" t="inlineStr"/>
+      <c r="E315" t="n">
+        <v>0</v>
+      </c>
+      <c r="F315" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="316">
       <c r="A316" t="inlineStr">
@@ -7308,7 +7891,12 @@
       <c r="D316" s="1" t="n">
         <v>46190</v>
       </c>
-      <c r="E316" t="inlineStr"/>
+      <c r="E316" t="n">
+        <v>0</v>
+      </c>
+      <c r="F316" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="317">
       <c r="A317" t="inlineStr">
@@ -7329,7 +7917,12 @@
       <c r="D317" s="1" t="n">
         <v>46190</v>
       </c>
-      <c r="E317" t="inlineStr"/>
+      <c r="E317" t="n">
+        <v>0</v>
+      </c>
+      <c r="F317" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="318">
       <c r="A318" t="inlineStr">
@@ -7350,7 +7943,12 @@
       <c r="D318" s="1" t="n">
         <v>46191</v>
       </c>
-      <c r="E318" t="inlineStr"/>
+      <c r="E318" t="n">
+        <v>5</v>
+      </c>
+      <c r="F318" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="319">
       <c r="A319" t="inlineStr">
@@ -7371,7 +7969,12 @@
       <c r="D319" s="1" t="n">
         <v>46191</v>
       </c>
-      <c r="E319" t="inlineStr"/>
+      <c r="E319" t="n">
+        <v>0</v>
+      </c>
+      <c r="F319" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="320">
       <c r="A320" t="inlineStr">
@@ -7392,7 +7995,12 @@
       <c r="D320" s="1" t="n">
         <v>46191</v>
       </c>
-      <c r="E320" t="inlineStr"/>
+      <c r="E320" t="n">
+        <v>0</v>
+      </c>
+      <c r="F320" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="321">
       <c r="A321" t="inlineStr">
@@ -7413,7 +8021,12 @@
       <c r="D321" s="1" t="n">
         <v>46191</v>
       </c>
-      <c r="E321" t="inlineStr"/>
+      <c r="E321" t="n">
+        <v>0</v>
+      </c>
+      <c r="F321" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="322">
       <c r="A322" t="inlineStr">
@@ -7434,7 +8047,12 @@
       <c r="D322" s="1" t="n">
         <v>46192</v>
       </c>
-      <c r="E322" t="inlineStr"/>
+      <c r="E322" t="n">
+        <v>6</v>
+      </c>
+      <c r="F322" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="323">
       <c r="A323" t="inlineStr">
@@ -7455,7 +8073,12 @@
       <c r="D323" s="1" t="n">
         <v>46192</v>
       </c>
-      <c r="E323" t="inlineStr"/>
+      <c r="E323" t="n">
+        <v>0</v>
+      </c>
+      <c r="F323" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="324">
       <c r="A324" t="inlineStr">
@@ -7476,7 +8099,12 @@
       <c r="D324" s="1" t="n">
         <v>46192</v>
       </c>
-      <c r="E324" t="inlineStr"/>
+      <c r="E324" t="n">
+        <v>0</v>
+      </c>
+      <c r="F324" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="325">
       <c r="A325" t="inlineStr">
@@ -7497,7 +8125,12 @@
       <c r="D325" s="1" t="n">
         <v>46192</v>
       </c>
-      <c r="E325" t="inlineStr"/>
+      <c r="E325" t="n">
+        <v>0</v>
+      </c>
+      <c r="F325" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="326">
       <c r="A326" t="inlineStr">
@@ -7518,7 +8151,12 @@
       <c r="D326" s="1" t="n">
         <v>46193</v>
       </c>
-      <c r="E326" t="inlineStr"/>
+      <c r="E326" t="n">
+        <v>7</v>
+      </c>
+      <c r="F326" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="327">
       <c r="A327" t="inlineStr">
@@ -7539,7 +8177,12 @@
       <c r="D327" s="1" t="n">
         <v>46193</v>
       </c>
-      <c r="E327" t="inlineStr"/>
+      <c r="E327" t="n">
+        <v>0</v>
+      </c>
+      <c r="F327" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="328">
       <c r="A328" t="inlineStr">
@@ -7560,7 +8203,12 @@
       <c r="D328" s="1" t="n">
         <v>46193</v>
       </c>
-      <c r="E328" t="inlineStr"/>
+      <c r="E328" t="n">
+        <v>0</v>
+      </c>
+      <c r="F328" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="329">
       <c r="A329" t="inlineStr">
@@ -7581,7 +8229,12 @@
       <c r="D329" s="1" t="n">
         <v>46193</v>
       </c>
-      <c r="E329" t="inlineStr"/>
+      <c r="E329" t="n">
+        <v>0</v>
+      </c>
+      <c r="F329" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="330">
       <c r="A330" t="inlineStr">
@@ -7596,13 +8249,18 @@
       </c>
       <c r="C330" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="D330" s="1" t="n">
         <v>46194</v>
       </c>
-      <c r="E330" t="inlineStr"/>
+      <c r="E330" t="n">
+        <v>0</v>
+      </c>
+      <c r="F330" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="331">
       <c r="A331" t="inlineStr">
@@ -7617,13 +8275,18 @@
       </c>
       <c r="C331" t="inlineStr">
         <is>
-          <t>T2</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="D331" s="1" t="n">
         <v>46194</v>
       </c>
-      <c r="E331" t="inlineStr"/>
+      <c r="E331" t="n">
+        <v>1</v>
+      </c>
+      <c r="F331" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="332">
       <c r="A332" t="inlineStr">
@@ -7644,7 +8307,12 @@
       <c r="D332" s="1" t="n">
         <v>46194</v>
       </c>
-      <c r="E332" t="inlineStr"/>
+      <c r="E332" t="n">
+        <v>0</v>
+      </c>
+      <c r="F332" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="333">
       <c r="A333" t="inlineStr">
@@ -7665,7 +8333,12 @@
       <c r="D333" s="1" t="n">
         <v>46194</v>
       </c>
-      <c r="E333" t="inlineStr"/>
+      <c r="E333" t="n">
+        <v>0</v>
+      </c>
+      <c r="F333" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="334">
       <c r="A334" t="inlineStr">
@@ -7680,13 +8353,18 @@
       </c>
       <c r="C334" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>COMP</t>
         </is>
       </c>
       <c r="D334" s="1" t="n">
         <v>46195</v>
       </c>
-      <c r="E334" t="inlineStr"/>
+      <c r="E334" t="n">
+        <v>0</v>
+      </c>
+      <c r="F334" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="335">
       <c r="A335" t="inlineStr">
@@ -7701,13 +8379,18 @@
       </c>
       <c r="C335" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="D335" s="1" t="n">
         <v>46195</v>
       </c>
-      <c r="E335" t="inlineStr"/>
+      <c r="E335" t="n">
+        <v>2</v>
+      </c>
+      <c r="F335" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="336">
       <c r="A336" t="inlineStr">
@@ -7722,13 +8405,18 @@
       </c>
       <c r="C336" t="inlineStr">
         <is>
-          <t>COMP</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="D336" s="1" t="n">
         <v>46195</v>
       </c>
-      <c r="E336" t="inlineStr"/>
+      <c r="E336" t="n">
+        <v>0</v>
+      </c>
+      <c r="F336" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="337">
       <c r="A337" t="inlineStr">
@@ -7749,7 +8437,12 @@
       <c r="D337" s="1" t="n">
         <v>46195</v>
       </c>
-      <c r="E337" t="inlineStr"/>
+      <c r="E337" t="n">
+        <v>0</v>
+      </c>
+      <c r="F337" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="338">
       <c r="A338" t="inlineStr">
@@ -7764,13 +8457,18 @@
       </c>
       <c r="C338" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>COMP</t>
         </is>
       </c>
       <c r="D338" s="1" t="n">
         <v>46196</v>
       </c>
-      <c r="E338" t="inlineStr"/>
+      <c r="E338" t="n">
+        <v>0</v>
+      </c>
+      <c r="F338" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="339">
       <c r="A339" t="inlineStr">
@@ -7785,13 +8483,18 @@
       </c>
       <c r="C339" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="D339" s="1" t="n">
         <v>46196</v>
       </c>
-      <c r="E339" t="inlineStr"/>
+      <c r="E339" t="n">
+        <v>3</v>
+      </c>
+      <c r="F339" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="340">
       <c r="A340" t="inlineStr">
@@ -7806,13 +8509,18 @@
       </c>
       <c r="C340" t="inlineStr">
         <is>
-          <t>T2</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="D340" s="1" t="n">
         <v>46196</v>
       </c>
-      <c r="E340" t="inlineStr"/>
+      <c r="E340" t="n">
+        <v>0</v>
+      </c>
+      <c r="F340" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="341">
       <c r="A341" t="inlineStr">
@@ -7833,7 +8541,12 @@
       <c r="D341" s="1" t="n">
         <v>46196</v>
       </c>
-      <c r="E341" t="inlineStr"/>
+      <c r="E341" t="n">
+        <v>0</v>
+      </c>
+      <c r="F341" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="342">
       <c r="A342" t="inlineStr">
@@ -7848,13 +8561,18 @@
       </c>
       <c r="C342" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="D342" s="1" t="n">
         <v>46197</v>
       </c>
-      <c r="E342" t="inlineStr"/>
+      <c r="E342" t="n">
+        <v>0</v>
+      </c>
+      <c r="F342" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="343">
       <c r="A343" t="inlineStr">
@@ -7869,13 +8587,18 @@
       </c>
       <c r="C343" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="D343" s="1" t="n">
         <v>46197</v>
       </c>
-      <c r="E343" t="inlineStr"/>
+      <c r="E343" t="n">
+        <v>4</v>
+      </c>
+      <c r="F343" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="344">
       <c r="A344" t="inlineStr">
@@ -7890,13 +8613,18 @@
       </c>
       <c r="C344" t="inlineStr">
         <is>
-          <t>T2</t>
+          <t>COMP</t>
         </is>
       </c>
       <c r="D344" s="1" t="n">
         <v>46197</v>
       </c>
-      <c r="E344" t="inlineStr"/>
+      <c r="E344" t="n">
+        <v>0</v>
+      </c>
+      <c r="F344" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="345">
       <c r="A345" t="inlineStr">
@@ -7917,7 +8645,12 @@
       <c r="D345" s="1" t="n">
         <v>46197</v>
       </c>
-      <c r="E345" t="inlineStr"/>
+      <c r="E345" t="n">
+        <v>0</v>
+      </c>
+      <c r="F345" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="346">
       <c r="A346" t="inlineStr">
@@ -7932,13 +8665,18 @@
       </c>
       <c r="C346" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="D346" s="1" t="n">
         <v>46198</v>
       </c>
-      <c r="E346" t="inlineStr"/>
+      <c r="E346" t="n">
+        <v>0</v>
+      </c>
+      <c r="F346" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="347">
       <c r="A347" t="inlineStr">
@@ -7953,13 +8691,18 @@
       </c>
       <c r="C347" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="D347" s="1" t="n">
         <v>46198</v>
       </c>
-      <c r="E347" t="inlineStr"/>
+      <c r="E347" t="n">
+        <v>5</v>
+      </c>
+      <c r="F347" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="348">
       <c r="A348" t="inlineStr">
@@ -7980,7 +8723,12 @@
       <c r="D348" s="1" t="n">
         <v>46198</v>
       </c>
-      <c r="E348" t="inlineStr"/>
+      <c r="E348" t="n">
+        <v>0</v>
+      </c>
+      <c r="F348" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="349">
       <c r="A349" t="inlineStr">
@@ -8001,7 +8749,12 @@
       <c r="D349" s="1" t="n">
         <v>46198</v>
       </c>
-      <c r="E349" t="inlineStr"/>
+      <c r="E349" t="n">
+        <v>0</v>
+      </c>
+      <c r="F349" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="350">
       <c r="A350" t="inlineStr">
@@ -8016,13 +8769,18 @@
       </c>
       <c r="C350" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="D350" s="1" t="n">
         <v>46199</v>
       </c>
-      <c r="E350" t="inlineStr"/>
+      <c r="E350" t="n">
+        <v>0</v>
+      </c>
+      <c r="F350" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="351">
       <c r="A351" t="inlineStr">
@@ -8037,13 +8795,18 @@
       </c>
       <c r="C351" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="D351" s="1" t="n">
         <v>46199</v>
       </c>
-      <c r="E351" t="inlineStr"/>
+      <c r="E351" t="n">
+        <v>6</v>
+      </c>
+      <c r="F351" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="352">
       <c r="A352" t="inlineStr">
@@ -8064,7 +8827,12 @@
       <c r="D352" s="1" t="n">
         <v>46199</v>
       </c>
-      <c r="E352" t="inlineStr"/>
+      <c r="E352" t="n">
+        <v>0</v>
+      </c>
+      <c r="F352" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="353">
       <c r="A353" t="inlineStr">
@@ -8085,7 +8853,12 @@
       <c r="D353" s="1" t="n">
         <v>46199</v>
       </c>
-      <c r="E353" t="inlineStr"/>
+      <c r="E353" t="n">
+        <v>0</v>
+      </c>
+      <c r="F353" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="354">
       <c r="A354" t="inlineStr">
@@ -8106,7 +8879,12 @@
       <c r="D354" s="1" t="n">
         <v>46200</v>
       </c>
-      <c r="E354" t="inlineStr"/>
+      <c r="E354" t="n">
+        <v>0</v>
+      </c>
+      <c r="F354" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="355">
       <c r="A355" t="inlineStr">
@@ -8127,7 +8905,12 @@
       <c r="D355" s="1" t="n">
         <v>46200</v>
       </c>
-      <c r="E355" t="inlineStr"/>
+      <c r="E355" t="n">
+        <v>0</v>
+      </c>
+      <c r="F355" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="356">
       <c r="A356" t="inlineStr">
@@ -8148,7 +8931,12 @@
       <c r="D356" s="1" t="n">
         <v>46200</v>
       </c>
-      <c r="E356" t="inlineStr"/>
+      <c r="E356" t="n">
+        <v>0</v>
+      </c>
+      <c r="F356" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="357">
       <c r="A357" t="inlineStr">
@@ -8169,7 +8957,12 @@
       <c r="D357" s="1" t="n">
         <v>46200</v>
       </c>
-      <c r="E357" t="inlineStr"/>
+      <c r="E357" t="n">
+        <v>1</v>
+      </c>
+      <c r="F357" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="358">
       <c r="A358" t="inlineStr">
@@ -8190,7 +8983,12 @@
       <c r="D358" s="1" t="n">
         <v>46201</v>
       </c>
-      <c r="E358" t="inlineStr"/>
+      <c r="E358" t="n">
+        <v>0</v>
+      </c>
+      <c r="F358" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="359">
       <c r="A359" t="inlineStr">
@@ -8211,7 +9009,12 @@
       <c r="D359" s="1" t="n">
         <v>46201</v>
       </c>
-      <c r="E359" t="inlineStr"/>
+      <c r="E359" t="n">
+        <v>0</v>
+      </c>
+      <c r="F359" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="360">
       <c r="A360" t="inlineStr">
@@ -8232,7 +9035,12 @@
       <c r="D360" s="1" t="n">
         <v>46201</v>
       </c>
-      <c r="E360" t="inlineStr"/>
+      <c r="E360" t="n">
+        <v>0</v>
+      </c>
+      <c r="F360" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="361">
       <c r="A361" t="inlineStr">
@@ -8253,7 +9061,12 @@
       <c r="D361" s="1" t="n">
         <v>46201</v>
       </c>
-      <c r="E361" t="inlineStr"/>
+      <c r="E361" t="n">
+        <v>2</v>
+      </c>
+      <c r="F361" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="362">
       <c r="A362" t="inlineStr">
@@ -8268,13 +9081,18 @@
       </c>
       <c r="C362" t="inlineStr">
         <is>
-          <t>COMP</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="D362" s="1" t="n">
         <v>46202</v>
       </c>
-      <c r="E362" t="inlineStr"/>
+      <c r="E362" t="n">
+        <v>0</v>
+      </c>
+      <c r="F362" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="363">
       <c r="A363" t="inlineStr">
@@ -8289,13 +9107,18 @@
       </c>
       <c r="C363" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>COMP</t>
         </is>
       </c>
       <c r="D363" s="1" t="n">
         <v>46202</v>
       </c>
-      <c r="E363" t="inlineStr"/>
+      <c r="E363" t="n">
+        <v>0</v>
+      </c>
+      <c r="F363" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="364">
       <c r="A364" t="inlineStr">
@@ -8316,7 +9139,12 @@
       <c r="D364" s="1" t="n">
         <v>46202</v>
       </c>
-      <c r="E364" t="inlineStr"/>
+      <c r="E364" t="n">
+        <v>0</v>
+      </c>
+      <c r="F364" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="365">
       <c r="A365" t="inlineStr">
@@ -8337,7 +9165,12 @@
       <c r="D365" s="1" t="n">
         <v>46202</v>
       </c>
-      <c r="E365" t="inlineStr"/>
+      <c r="E365" t="n">
+        <v>3</v>
+      </c>
+      <c r="F365" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="366">
       <c r="A366" t="inlineStr">
@@ -8352,13 +9185,18 @@
       </c>
       <c r="C366" t="inlineStr">
         <is>
-          <t>COMP</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="D366" s="1" t="n">
         <v>46203</v>
       </c>
-      <c r="E366" t="inlineStr"/>
+      <c r="E366" t="n">
+        <v>0</v>
+      </c>
+      <c r="F366" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="367">
       <c r="A367" t="inlineStr">
@@ -8373,13 +9211,18 @@
       </c>
       <c r="C367" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="D367" s="1" t="n">
         <v>46203</v>
       </c>
-      <c r="E367" t="inlineStr"/>
+      <c r="E367" t="n">
+        <v>0</v>
+      </c>
+      <c r="F367" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="368">
       <c r="A368" t="inlineStr">
@@ -8400,7 +9243,12 @@
       <c r="D368" s="1" t="n">
         <v>46203</v>
       </c>
-      <c r="E368" t="inlineStr"/>
+      <c r="E368" t="n">
+        <v>0</v>
+      </c>
+      <c r="F368" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="369">
       <c r="A369" t="inlineStr">
@@ -8421,7 +9269,12 @@
       <c r="D369" s="1" t="n">
         <v>46203</v>
       </c>
-      <c r="E369" t="inlineStr"/>
+      <c r="E369" t="n">
+        <v>4</v>
+      </c>
+      <c r="F369" t="n">
+        <v>1</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Malla Refuerzo T2 Final
</commit_message>
<xml_diff>
--- a/malla_historica.xlsx
+++ b/malla_historica.xlsx
@@ -6169,14 +6169,14 @@
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="D250" s="1" t="n">
         <v>46174</v>
       </c>
       <c r="E250" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F250" t="n">
         <v>0</v>
@@ -6273,14 +6273,14 @@
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="D254" s="1" t="n">
         <v>46175</v>
       </c>
       <c r="E254" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F254" t="n">
         <v>0</v>
@@ -6377,14 +6377,14 @@
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="D258" s="1" t="n">
         <v>46176</v>
       </c>
       <c r="E258" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F258" t="n">
         <v>0</v>
@@ -6481,14 +6481,14 @@
       </c>
       <c r="C262" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="D262" s="1" t="n">
         <v>46177</v>
       </c>
       <c r="E262" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F262" t="n">
         <v>0</v>
@@ -6585,14 +6585,14 @@
       </c>
       <c r="C266" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="D266" s="1" t="n">
         <v>46178</v>
       </c>
       <c r="E266" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="F266" t="n">
         <v>0</v>
@@ -6689,14 +6689,14 @@
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="D270" s="1" t="n">
         <v>46179</v>
       </c>
       <c r="E270" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="F270" t="n">
         <v>1</v>
@@ -6793,14 +6793,14 @@
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="D274" s="1" t="n">
         <v>46180</v>
       </c>
       <c r="E274" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F274" t="n">
         <v>1</v>
@@ -6819,14 +6819,14 @@
       </c>
       <c r="C275" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="D275" s="1" t="n">
         <v>46180</v>
       </c>
       <c r="E275" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F275" t="n">
         <v>0</v>
@@ -6897,17 +6897,17 @@
       </c>
       <c r="C278" t="inlineStr">
         <is>
-          <t>COMP</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="D278" s="1" t="n">
         <v>46181</v>
       </c>
       <c r="E278" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F278" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="279">
@@ -6923,14 +6923,14 @@
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="D279" s="1" t="n">
         <v>46181</v>
       </c>
       <c r="E279" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F279" t="n">
         <v>0</v>
@@ -6949,7 +6949,7 @@
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>T2</t>
+          <t>COMP</t>
         </is>
       </c>
       <c r="D280" s="1" t="n">
@@ -6959,7 +6959,7 @@
         <v>0</v>
       </c>
       <c r="F280" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="281">
@@ -7001,17 +7001,17 @@
       </c>
       <c r="C282" t="inlineStr">
         <is>
-          <t>T2</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="D282" s="1" t="n">
         <v>46182</v>
       </c>
       <c r="E282" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F282" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="283">
@@ -7027,14 +7027,14 @@
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="D283" s="1" t="n">
         <v>46182</v>
       </c>
       <c r="E283" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F283" t="n">
         <v>0</v>
@@ -7053,7 +7053,7 @@
       </c>
       <c r="C284" t="inlineStr">
         <is>
-          <t>COMP</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="D284" s="1" t="n">
@@ -7105,17 +7105,17 @@
       </c>
       <c r="C286" t="inlineStr">
         <is>
-          <t>T2</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="D286" s="1" t="n">
         <v>46183</v>
       </c>
       <c r="E286" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F286" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="287">
@@ -7131,14 +7131,14 @@
       </c>
       <c r="C287" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="D287" s="1" t="n">
         <v>46183</v>
       </c>
       <c r="E287" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F287" t="n">
         <v>0</v>
@@ -7157,14 +7157,14 @@
       </c>
       <c r="C288" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="D288" s="1" t="n">
         <v>46183</v>
       </c>
       <c r="E288" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F288" t="n">
         <v>0</v>
@@ -7209,17 +7209,17 @@
       </c>
       <c r="C290" t="inlineStr">
         <is>
-          <t>T2</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="D290" s="1" t="n">
         <v>46184</v>
       </c>
       <c r="E290" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="F290" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="291">
@@ -7235,14 +7235,14 @@
       </c>
       <c r="C291" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="D291" s="1" t="n">
         <v>46184</v>
       </c>
       <c r="E291" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="F291" t="n">
         <v>0</v>
@@ -7261,14 +7261,14 @@
       </c>
       <c r="C292" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="D292" s="1" t="n">
         <v>46184</v>
       </c>
       <c r="E292" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F292" t="n">
         <v>0</v>
@@ -7313,17 +7313,17 @@
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>T2</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="D294" s="1" t="n">
         <v>46185</v>
       </c>
       <c r="E294" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="F294" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="295">
@@ -7339,14 +7339,14 @@
       </c>
       <c r="C295" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="D295" s="1" t="n">
         <v>46185</v>
       </c>
       <c r="E295" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="F295" t="n">
         <v>0</v>
@@ -7365,14 +7365,14 @@
       </c>
       <c r="C296" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="D296" s="1" t="n">
         <v>46185</v>
       </c>
       <c r="E296" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F296" t="n">
         <v>0</v>
@@ -7427,7 +7427,7 @@
         <v>0</v>
       </c>
       <c r="F298" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="299">
@@ -7443,7 +7443,7 @@
       </c>
       <c r="C299" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="D299" s="1" t="n">
@@ -7476,7 +7476,7 @@
         <v>46186</v>
       </c>
       <c r="E300" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F300" t="n">
         <v>0</v>
@@ -7495,7 +7495,7 @@
       </c>
       <c r="C301" t="inlineStr">
         <is>
-          <t>T2</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="D301" s="1" t="n">
@@ -7531,7 +7531,7 @@
         <v>1</v>
       </c>
       <c r="F302" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="303">
@@ -7635,7 +7635,7 @@
         <v>2</v>
       </c>
       <c r="F306" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="307">
@@ -7739,7 +7739,7 @@
         <v>3</v>
       </c>
       <c r="F310" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="311">
@@ -7843,7 +7843,7 @@
         <v>4</v>
       </c>
       <c r="F314" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="315">
@@ -7859,14 +7859,14 @@
       </c>
       <c r="C315" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="D315" s="1" t="n">
         <v>46190</v>
       </c>
       <c r="E315" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F315" t="n">
         <v>0</v>
@@ -7947,7 +7947,7 @@
         <v>5</v>
       </c>
       <c r="F318" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="319">
@@ -7963,14 +7963,14 @@
       </c>
       <c r="C319" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="D319" s="1" t="n">
         <v>46191</v>
       </c>
       <c r="E319" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F319" t="n">
         <v>0</v>
@@ -8051,7 +8051,7 @@
         <v>6</v>
       </c>
       <c r="F322" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="323">
@@ -8067,14 +8067,14 @@
       </c>
       <c r="C323" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="D323" s="1" t="n">
         <v>46192</v>
       </c>
       <c r="E323" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F323" t="n">
         <v>0</v>
@@ -8155,7 +8155,7 @@
         <v>0</v>
       </c>
       <c r="F326" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="327">
@@ -8259,7 +8259,7 @@
         <v>0</v>
       </c>
       <c r="F330" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="331">
@@ -8363,7 +8363,7 @@
         <v>0</v>
       </c>
       <c r="F334" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="335">
@@ -8457,7 +8457,7 @@
       </c>
       <c r="C338" t="inlineStr">
         <is>
-          <t>T2</t>
+          <t>COMP</t>
         </is>
       </c>
       <c r="D338" s="1" t="n">
@@ -8535,14 +8535,14 @@
       </c>
       <c r="C341" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="D341" s="1" t="n">
         <v>46196</v>
       </c>
       <c r="E341" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F341" t="n">
         <v>0</v>
@@ -8639,14 +8639,14 @@
       </c>
       <c r="C345" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="D345" s="1" t="n">
         <v>46197</v>
       </c>
       <c r="E345" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F345" t="n">
         <v>0</v>
@@ -8743,14 +8743,14 @@
       </c>
       <c r="C349" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="D349" s="1" t="n">
         <v>46198</v>
       </c>
       <c r="E349" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F349" t="n">
         <v>0</v>
@@ -8795,7 +8795,7 @@
       </c>
       <c r="C351" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="D351" s="1" t="n">
@@ -8854,7 +8854,7 @@
         <v>46199</v>
       </c>
       <c r="E353" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F353" t="n">
         <v>0</v>
@@ -8958,7 +8958,7 @@
         <v>46200</v>
       </c>
       <c r="E357" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F357" t="n">
         <v>0</v>
@@ -9062,7 +9062,7 @@
         <v>46201</v>
       </c>
       <c r="E361" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F361" t="n">
         <v>1</v>
@@ -9081,7 +9081,7 @@
       </c>
       <c r="C362" t="inlineStr">
         <is>
-          <t>T2</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="D362" s="1" t="n">
@@ -9133,14 +9133,14 @@
       </c>
       <c r="C364" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="D364" s="1" t="n">
         <v>46202</v>
       </c>
       <c r="E364" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F364" t="n">
         <v>1</v>
@@ -9159,14 +9159,14 @@
       </c>
       <c r="C365" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="D365" s="1" t="n">
         <v>46202</v>
       </c>
       <c r="E365" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F365" t="n">
         <v>1</v>
@@ -9237,17 +9237,17 @@
       </c>
       <c r="C368" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>COMP</t>
         </is>
       </c>
       <c r="D368" s="1" t="n">
         <v>46203</v>
       </c>
       <c r="E368" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F368" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="369">
@@ -9263,17 +9263,17 @@
       </c>
       <c r="C369" t="inlineStr">
         <is>
-          <t>COMP</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="D369" s="1" t="n">
         <v>46203</v>
       </c>
       <c r="E369" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="F369" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Malla Saludable Richard V4
</commit_message>
<xml_diff>
--- a/malla_historica.xlsx
+++ b/malla_historica.xlsx
@@ -54113,7 +54113,7 @@
       </c>
       <c r="C1586" t="inlineStr">
         <is>
-          <t>T2</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="D1586" s="1" t="n">
@@ -54249,7 +54249,7 @@
       </c>
       <c r="C1590" t="inlineStr">
         <is>
-          <t>T2</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="D1590" s="1" t="n">
@@ -54385,7 +54385,7 @@
       </c>
       <c r="C1594" t="inlineStr">
         <is>
-          <t>T2</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="D1594" s="1" t="n">
@@ -54521,7 +54521,7 @@
       </c>
       <c r="C1598" t="inlineStr">
         <is>
-          <t>T2</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="D1598" s="1" t="n">
@@ -54657,7 +54657,7 @@
       </c>
       <c r="C1602" t="inlineStr">
         <is>
-          <t>T2</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="D1602" s="1" t="n">
@@ -54793,7 +54793,7 @@
       </c>
       <c r="C1606" t="inlineStr">
         <is>
-          <t>T2</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="D1606" s="1" t="n">
@@ -55201,7 +55201,7 @@
       </c>
       <c r="C1618" t="inlineStr">
         <is>
-          <t>T2</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="D1618" s="1" t="n">
@@ -56289,7 +56289,7 @@
       </c>
       <c r="C1650" t="inlineStr">
         <is>
-          <t>T2</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="D1650" s="1" t="n">
@@ -56425,7 +56425,7 @@
       </c>
       <c r="C1654" t="inlineStr">
         <is>
-          <t>T2</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="D1654" s="1" t="n">
@@ -56561,7 +56561,7 @@
       </c>
       <c r="C1658" t="inlineStr">
         <is>
-          <t>T2</t>
+          <t>DESC</t>
         </is>
       </c>
       <c r="D1658" s="1" t="n">
@@ -56697,7 +56697,7 @@
       </c>
       <c r="C1662" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>DESC</t>
         </is>
       </c>
       <c r="D1662" s="1" t="n">
@@ -56731,7 +56731,7 @@
       </c>
       <c r="C1663" t="inlineStr">
         <is>
-          <t>DESC</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="D1663" s="1" t="n">
@@ -56867,7 +56867,7 @@
       </c>
       <c r="C1667" t="inlineStr">
         <is>
-          <t>T2</t>
+          <t>COMP</t>
         </is>
       </c>
       <c r="D1667" s="1" t="n">
@@ -57105,7 +57105,7 @@
       </c>
       <c r="C1674" t="inlineStr">
         <is>
-          <t>T2</t>
+          <t>COMP</t>
         </is>
       </c>
       <c r="D1674" s="1" t="n">
@@ -57241,7 +57241,7 @@
       </c>
       <c r="C1678" t="inlineStr">
         <is>
-          <t>COMP</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="D1678" s="1" t="n">

</xml_diff>

<commit_message>
Malla V7.0 - Cobertura Garantizada
</commit_message>
<xml_diff>
--- a/malla_historica.xlsx
+++ b/malla_historica.xlsx
@@ -2738,7 +2738,7 @@
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>T2</t>
+          <t>T3</t>
         </is>
       </c>
     </row>
@@ -2773,7 +2773,7 @@
       </c>
       <c r="I67" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T1</t>
         </is>
       </c>
     </row>
@@ -2808,7 +2808,7 @@
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T2</t>
         </is>
       </c>
     </row>
@@ -3333,7 +3333,7 @@
       </c>
       <c r="I83" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T3</t>
         </is>
       </c>
     </row>
@@ -3473,7 +3473,7 @@
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>T2</t>
+          <t>COMP</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización Malla con Validadores
</commit_message>
<xml_diff>
--- a/malla_historica.xlsx
+++ b/malla_historica.xlsx
@@ -508,11 +508,11 @@
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K2" t="n">
         <v>2</v>
@@ -656,11 +656,11 @@
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J6" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K6" t="n">
         <v>2</v>
@@ -804,11 +804,11 @@
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J10" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K10" t="n">
         <v>2</v>
@@ -915,7 +915,7 @@
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>DESC</t>
         </is>
       </c>
       <c r="J13" t="n">
@@ -952,7 +952,7 @@
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr">
         <is>
-          <t>DESC</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="J14" t="n">
@@ -1100,11 +1100,11 @@
       <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="J18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K18" t="n">
         <v>2</v>
@@ -1211,7 +1211,7 @@
       <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr">
         <is>
-          <t>DESC</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J21" t="n">
@@ -1248,7 +1248,7 @@
       <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr">
         <is>
-          <t>T2</t>
+          <t>DESC</t>
         </is>
       </c>
       <c r="J22" t="n">
@@ -1951,7 +1951,7 @@
       <c r="H41" t="inlineStr"/>
       <c r="I41" t="inlineStr">
         <is>
-          <t>T2</t>
+          <t>DESC</t>
         </is>
       </c>
       <c r="J41" t="n">
@@ -1988,11 +1988,11 @@
       <c r="H42" t="inlineStr"/>
       <c r="I42" t="inlineStr">
         <is>
-          <t>DESC</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="J42" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K42" t="n">
         <v>2</v>
@@ -2136,11 +2136,11 @@
       <c r="H46" t="inlineStr"/>
       <c r="I46" t="inlineStr">
         <is>
-          <t>T2</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="J46" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K46" t="n">
         <v>2</v>
@@ -2173,11 +2173,11 @@
       <c r="H47" t="inlineStr"/>
       <c r="I47" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J47" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K47" t="n">
         <v>2</v>
@@ -2247,7 +2247,7 @@
       <c r="H49" t="inlineStr"/>
       <c r="I49" t="inlineStr">
         <is>
-          <t>DESC</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="J49" t="n">
@@ -2284,11 +2284,11 @@
       <c r="H50" t="inlineStr"/>
       <c r="I50" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>DESC</t>
         </is>
       </c>
       <c r="J50" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K50" t="n">
         <v>2</v>
@@ -2321,11 +2321,11 @@
       <c r="H51" t="inlineStr"/>
       <c r="I51" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J51" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K51" t="n">
         <v>2</v>
@@ -2395,11 +2395,11 @@
       <c r="H53" t="inlineStr"/>
       <c r="I53" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="J53" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K53" t="n">
         <v>2</v>
@@ -2436,7 +2436,7 @@
         </is>
       </c>
       <c r="J54" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K54" t="n">
         <v>2</v>
@@ -2469,11 +2469,11 @@
       <c r="H55" t="inlineStr"/>
       <c r="I55" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J55" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K55" t="n">
         <v>2</v>
@@ -2543,11 +2543,11 @@
       <c r="H57" t="inlineStr"/>
       <c r="I57" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="J57" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K57" t="n">
         <v>2</v>
@@ -2584,7 +2584,7 @@
         </is>
       </c>
       <c r="J58" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K58" t="n">
         <v>2</v>
@@ -2617,11 +2617,11 @@
       <c r="H59" t="inlineStr"/>
       <c r="I59" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J59" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="K59" t="n">
         <v>2</v>
@@ -2691,11 +2691,11 @@
       <c r="H61" t="inlineStr"/>
       <c r="I61" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="J61" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K61" t="n">
         <v>2</v>
@@ -2732,7 +2732,7 @@
         </is>
       </c>
       <c r="J62" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K62" t="n">
         <v>2</v>
@@ -2765,11 +2765,11 @@
       <c r="H63" t="inlineStr"/>
       <c r="I63" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J63" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="K63" t="n">
         <v>2</v>
@@ -2839,11 +2839,11 @@
       <c r="H65" t="inlineStr"/>
       <c r="I65" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="J65" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="K65" t="n">
         <v>2</v>
@@ -2880,7 +2880,7 @@
         </is>
       </c>
       <c r="J66" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K66" t="n">
         <v>2</v>
@@ -2913,11 +2913,11 @@
       <c r="H67" t="inlineStr"/>
       <c r="I67" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J67" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="K67" t="n">
         <v>2</v>
@@ -2987,7 +2987,7 @@
       <c r="H69" t="inlineStr"/>
       <c r="I69" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>DESC</t>
         </is>
       </c>
       <c r="J69" t="n">
@@ -3024,11 +3024,11 @@
       <c r="H70" t="inlineStr"/>
       <c r="I70" t="inlineStr">
         <is>
-          <t>DESC</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="J70" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="K70" t="n">
         <v>2</v>
@@ -3135,11 +3135,11 @@
       <c r="H73" t="inlineStr"/>
       <c r="I73" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J73" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K73" t="n">
         <v>2</v>
@@ -3176,7 +3176,7 @@
         </is>
       </c>
       <c r="J74" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="K74" t="n">
         <v>2</v>
@@ -3283,7 +3283,7 @@
       <c r="H77" t="inlineStr"/>
       <c r="I77" t="inlineStr">
         <is>
-          <t>DESC</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="J77" t="n">
@@ -3320,11 +3320,11 @@
       <c r="H78" t="inlineStr"/>
       <c r="I78" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>DESC</t>
         </is>
       </c>
       <c r="J78" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K78" t="n">
         <v>2</v>
@@ -3357,7 +3357,7 @@
       <c r="H79" t="inlineStr"/>
       <c r="I79" t="inlineStr">
         <is>
-          <t>T2</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J79" t="n">
@@ -3431,7 +3431,7 @@
       <c r="H81" t="inlineStr"/>
       <c r="I81" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="J81" t="n">
@@ -3468,11 +3468,11 @@
       <c r="H82" t="inlineStr"/>
       <c r="I82" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J82" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K82" t="n">
         <v>2</v>
@@ -3579,7 +3579,7 @@
       <c r="H85" t="inlineStr"/>
       <c r="I85" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="J85" t="n">
@@ -3616,11 +3616,11 @@
       <c r="H86" t="inlineStr"/>
       <c r="I86" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J86" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="K86" t="n">
         <v>2</v>
@@ -3727,7 +3727,7 @@
       <c r="H89" t="inlineStr"/>
       <c r="I89" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="J89" t="n">
@@ -3764,11 +3764,11 @@
       <c r="H90" t="inlineStr"/>
       <c r="I90" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J90" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="K90" t="n">
         <v>2</v>
@@ -3875,7 +3875,7 @@
       <c r="H93" t="inlineStr"/>
       <c r="I93" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="J93" t="n">
@@ -3912,11 +3912,11 @@
       <c r="H94" t="inlineStr"/>
       <c r="I94" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J94" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="K94" t="n">
         <v>2</v>
@@ -4023,7 +4023,7 @@
       <c r="H97" t="inlineStr"/>
       <c r="I97" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>DESC</t>
         </is>
       </c>
       <c r="J97" t="n">
@@ -4060,7 +4060,7 @@
       <c r="H98" t="inlineStr"/>
       <c r="I98" t="inlineStr">
         <is>
-          <t>DESC</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="J98" t="n">
@@ -4208,11 +4208,11 @@
       <c r="H102" t="inlineStr"/>
       <c r="I102" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="J102" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K102" t="n">
         <v>2</v>
@@ -4319,7 +4319,7 @@
       <c r="H105" t="inlineStr"/>
       <c r="I105" t="inlineStr">
         <is>
-          <t>DESC</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J105" t="n">
@@ -4356,7 +4356,7 @@
       <c r="H106" t="inlineStr"/>
       <c r="I106" t="inlineStr">
         <is>
-          <t>T2</t>
+          <t>DESC</t>
         </is>
       </c>
       <c r="J106" t="n">
@@ -5059,7 +5059,7 @@
       <c r="H125" t="inlineStr"/>
       <c r="I125" t="inlineStr">
         <is>
-          <t>T2</t>
+          <t>DESC</t>
         </is>
       </c>
       <c r="J125" t="n">
@@ -5096,11 +5096,11 @@
       <c r="H126" t="inlineStr"/>
       <c r="I126" t="inlineStr">
         <is>
-          <t>DESC</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="J126" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K126" t="n">
         <v>2</v>
@@ -5244,11 +5244,11 @@
       <c r="H130" t="inlineStr"/>
       <c r="I130" t="inlineStr">
         <is>
-          <t>T2</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="J130" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K130" t="n">
         <v>2</v>
@@ -5281,11 +5281,11 @@
       <c r="H131" t="inlineStr"/>
       <c r="I131" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J131" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K131" t="n">
         <v>2</v>
@@ -5355,7 +5355,7 @@
       <c r="H133" t="inlineStr"/>
       <c r="I133" t="inlineStr">
         <is>
-          <t>DESC</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="J133" t="n">
@@ -5392,11 +5392,11 @@
       <c r="H134" t="inlineStr"/>
       <c r="I134" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>DESC</t>
         </is>
       </c>
       <c r="J134" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K134" t="n">
         <v>2</v>
@@ -5429,11 +5429,11 @@
       <c r="H135" t="inlineStr"/>
       <c r="I135" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J135" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K135" t="n">
         <v>2</v>
@@ -5503,11 +5503,11 @@
       <c r="H137" t="inlineStr"/>
       <c r="I137" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="J137" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K137" t="n">
         <v>2</v>
@@ -5544,7 +5544,7 @@
         </is>
       </c>
       <c r="J138" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K138" t="n">
         <v>2</v>
@@ -5577,11 +5577,11 @@
       <c r="H139" t="inlineStr"/>
       <c r="I139" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J139" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K139" t="n">
         <v>2</v>
@@ -5651,11 +5651,11 @@
       <c r="H141" t="inlineStr"/>
       <c r="I141" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="J141" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K141" t="n">
         <v>2</v>
@@ -5692,7 +5692,7 @@
         </is>
       </c>
       <c r="J142" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K142" t="n">
         <v>2</v>
@@ -5725,11 +5725,11 @@
       <c r="H143" t="inlineStr"/>
       <c r="I143" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J143" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="K143" t="n">
         <v>2</v>
@@ -5799,11 +5799,11 @@
       <c r="H145" t="inlineStr"/>
       <c r="I145" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="J145" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K145" t="n">
         <v>2</v>
@@ -5840,7 +5840,7 @@
         </is>
       </c>
       <c r="J146" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K146" t="n">
         <v>2</v>
@@ -5873,11 +5873,11 @@
       <c r="H147" t="inlineStr"/>
       <c r="I147" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J147" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="K147" t="n">
         <v>2</v>
@@ -5947,11 +5947,11 @@
       <c r="H149" t="inlineStr"/>
       <c r="I149" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="J149" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="K149" t="n">
         <v>2</v>
@@ -5988,7 +5988,7 @@
         </is>
       </c>
       <c r="J150" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K150" t="n">
         <v>2</v>
@@ -6021,11 +6021,11 @@
       <c r="H151" t="inlineStr"/>
       <c r="I151" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J151" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="K151" t="n">
         <v>2</v>
@@ -6095,7 +6095,7 @@
       <c r="H153" t="inlineStr"/>
       <c r="I153" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>DESC</t>
         </is>
       </c>
       <c r="J153" t="n">
@@ -6132,11 +6132,11 @@
       <c r="H154" t="inlineStr"/>
       <c r="I154" t="inlineStr">
         <is>
-          <t>DESC</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="J154" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="K154" t="n">
         <v>2</v>
@@ -6243,11 +6243,11 @@
       <c r="H157" t="inlineStr"/>
       <c r="I157" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J157" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K157" t="n">
         <v>2</v>
@@ -6284,7 +6284,7 @@
         </is>
       </c>
       <c r="J158" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="K158" t="n">
         <v>2</v>
@@ -6391,7 +6391,7 @@
       <c r="H161" t="inlineStr"/>
       <c r="I161" t="inlineStr">
         <is>
-          <t>DESC</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="J161" t="n">
@@ -6428,11 +6428,11 @@
       <c r="H162" t="inlineStr"/>
       <c r="I162" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>DESC</t>
         </is>
       </c>
       <c r="J162" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K162" t="n">
         <v>2</v>
@@ -6465,7 +6465,7 @@
       <c r="H163" t="inlineStr"/>
       <c r="I163" t="inlineStr">
         <is>
-          <t>T2</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J163" t="n">
@@ -6539,7 +6539,7 @@
       <c r="H165" t="inlineStr"/>
       <c r="I165" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="J165" t="n">
@@ -6576,11 +6576,11 @@
       <c r="H166" t="inlineStr"/>
       <c r="I166" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J166" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K166" t="n">
         <v>2</v>
@@ -6687,7 +6687,7 @@
       <c r="H169" t="inlineStr"/>
       <c r="I169" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="J169" t="n">
@@ -6724,11 +6724,11 @@
       <c r="H170" t="inlineStr"/>
       <c r="I170" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J170" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="K170" t="n">
         <v>2</v>
@@ -6835,7 +6835,7 @@
       <c r="H173" t="inlineStr"/>
       <c r="I173" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="J173" t="n">
@@ -6872,11 +6872,11 @@
       <c r="H174" t="inlineStr"/>
       <c r="I174" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J174" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="K174" t="n">
         <v>2</v>
@@ -6983,7 +6983,7 @@
       <c r="H177" t="inlineStr"/>
       <c r="I177" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="J177" t="n">
@@ -7020,11 +7020,11 @@
       <c r="H178" t="inlineStr"/>
       <c r="I178" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J178" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="K178" t="n">
         <v>2</v>
@@ -7131,7 +7131,7 @@
       <c r="H181" t="inlineStr"/>
       <c r="I181" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>DESC</t>
         </is>
       </c>
       <c r="J181" t="n">
@@ -7168,7 +7168,7 @@
       <c r="H182" t="inlineStr"/>
       <c r="I182" t="inlineStr">
         <is>
-          <t>DESC</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="J182" t="n">
@@ -7316,11 +7316,11 @@
       <c r="H186" t="inlineStr"/>
       <c r="I186" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="J186" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K186" t="n">
         <v>2</v>
@@ -7427,7 +7427,7 @@
       <c r="H189" t="inlineStr"/>
       <c r="I189" t="inlineStr">
         <is>
-          <t>DESC</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J189" t="n">
@@ -7464,7 +7464,7 @@
       <c r="H190" t="inlineStr"/>
       <c r="I190" t="inlineStr">
         <is>
-          <t>T2</t>
+          <t>DESC</t>
         </is>
       </c>
       <c r="J190" t="n">
@@ -8167,7 +8167,7 @@
       <c r="H209" t="inlineStr"/>
       <c r="I209" t="inlineStr">
         <is>
-          <t>T2</t>
+          <t>DESC</t>
         </is>
       </c>
       <c r="J209" t="n">
@@ -8204,11 +8204,11 @@
       <c r="H210" t="inlineStr"/>
       <c r="I210" t="inlineStr">
         <is>
-          <t>DESC</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="J210" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K210" t="n">
         <v>2</v>
@@ -8352,11 +8352,11 @@
       <c r="H214" t="inlineStr"/>
       <c r="I214" t="inlineStr">
         <is>
-          <t>T2</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="J214" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K214" t="n">
         <v>2</v>
@@ -8389,11 +8389,11 @@
       <c r="H215" t="inlineStr"/>
       <c r="I215" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J215" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K215" t="n">
         <v>2</v>
@@ -8463,7 +8463,7 @@
       <c r="H217" t="inlineStr"/>
       <c r="I217" t="inlineStr">
         <is>
-          <t>DESC</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="J217" t="n">
@@ -8500,11 +8500,11 @@
       <c r="H218" t="inlineStr"/>
       <c r="I218" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>DESC</t>
         </is>
       </c>
       <c r="J218" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K218" t="n">
         <v>2</v>
@@ -8537,11 +8537,11 @@
       <c r="H219" t="inlineStr"/>
       <c r="I219" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J219" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K219" t="n">
         <v>2</v>
@@ -8611,11 +8611,11 @@
       <c r="H221" t="inlineStr"/>
       <c r="I221" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="J221" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K221" t="n">
         <v>2</v>
@@ -8652,7 +8652,7 @@
         </is>
       </c>
       <c r="J222" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K222" t="n">
         <v>2</v>
@@ -8685,11 +8685,11 @@
       <c r="H223" t="inlineStr"/>
       <c r="I223" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J223" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K223" t="n">
         <v>2</v>
@@ -8759,11 +8759,11 @@
       <c r="H225" t="inlineStr"/>
       <c r="I225" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="J225" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K225" t="n">
         <v>2</v>
@@ -8800,7 +8800,7 @@
         </is>
       </c>
       <c r="J226" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K226" t="n">
         <v>2</v>
@@ -8833,11 +8833,11 @@
       <c r="H227" t="inlineStr"/>
       <c r="I227" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J227" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="K227" t="n">
         <v>2</v>
@@ -8907,11 +8907,11 @@
       <c r="H229" t="inlineStr"/>
       <c r="I229" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="J229" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K229" t="n">
         <v>2</v>
@@ -8948,7 +8948,7 @@
         </is>
       </c>
       <c r="J230" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K230" t="n">
         <v>2</v>
@@ -8981,11 +8981,11 @@
       <c r="H231" t="inlineStr"/>
       <c r="I231" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J231" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="K231" t="n">
         <v>2</v>
@@ -9055,11 +9055,11 @@
       <c r="H233" t="inlineStr"/>
       <c r="I233" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="J233" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="K233" t="n">
         <v>2</v>
@@ -9096,7 +9096,7 @@
         </is>
       </c>
       <c r="J234" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K234" t="n">
         <v>2</v>
@@ -9129,11 +9129,11 @@
       <c r="H235" t="inlineStr"/>
       <c r="I235" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J235" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="K235" t="n">
         <v>2</v>
@@ -9203,7 +9203,7 @@
       <c r="H237" t="inlineStr"/>
       <c r="I237" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>DESC</t>
         </is>
       </c>
       <c r="J237" t="n">
@@ -9240,11 +9240,11 @@
       <c r="H238" t="inlineStr"/>
       <c r="I238" t="inlineStr">
         <is>
-          <t>DESC</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="J238" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="K238" t="n">
         <v>2</v>
@@ -9351,11 +9351,11 @@
       <c r="H241" t="inlineStr"/>
       <c r="I241" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J241" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K241" t="n">
         <v>2</v>
@@ -9392,7 +9392,7 @@
         </is>
       </c>
       <c r="J242" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="K242" t="n">
         <v>2</v>
@@ -9499,7 +9499,7 @@
       <c r="H245" t="inlineStr"/>
       <c r="I245" t="inlineStr">
         <is>
-          <t>DESC</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="J245" t="n">
@@ -9536,11 +9536,11 @@
       <c r="H246" t="inlineStr"/>
       <c r="I246" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>DESC</t>
         </is>
       </c>
       <c r="J246" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K246" t="n">
         <v>2</v>
@@ -9573,7 +9573,7 @@
       <c r="H247" t="inlineStr"/>
       <c r="I247" t="inlineStr">
         <is>
-          <t>T2</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J247" t="n">
@@ -9647,7 +9647,7 @@
       <c r="H249" t="inlineStr"/>
       <c r="I249" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="J249" t="n">
@@ -9684,11 +9684,11 @@
       <c r="H250" t="inlineStr"/>
       <c r="I250" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J250" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K250" t="n">
         <v>2</v>
@@ -9795,7 +9795,7 @@
       <c r="H253" t="inlineStr"/>
       <c r="I253" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="J253" t="n">
@@ -9832,11 +9832,11 @@
       <c r="H254" t="inlineStr"/>
       <c r="I254" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J254" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="K254" t="n">
         <v>2</v>
@@ -9943,7 +9943,7 @@
       <c r="H257" t="inlineStr"/>
       <c r="I257" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="J257" t="n">
@@ -9980,11 +9980,11 @@
       <c r="H258" t="inlineStr"/>
       <c r="I258" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J258" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="K258" t="n">
         <v>2</v>
@@ -10091,7 +10091,7 @@
       <c r="H261" t="inlineStr"/>
       <c r="I261" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="J261" t="n">
@@ -10128,11 +10128,11 @@
       <c r="H262" t="inlineStr"/>
       <c r="I262" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J262" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="K262" t="n">
         <v>2</v>
@@ -10239,7 +10239,7 @@
       <c r="H265" t="inlineStr"/>
       <c r="I265" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>DESC</t>
         </is>
       </c>
       <c r="J265" t="n">
@@ -10276,7 +10276,7 @@
       <c r="H266" t="inlineStr"/>
       <c r="I266" t="inlineStr">
         <is>
-          <t>DESC</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="J266" t="n">
@@ -10424,11 +10424,11 @@
       <c r="H270" t="inlineStr"/>
       <c r="I270" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="J270" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K270" t="n">
         <v>2</v>
@@ -10535,7 +10535,7 @@
       <c r="H273" t="inlineStr"/>
       <c r="I273" t="inlineStr">
         <is>
-          <t>DESC</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J273" t="n">
@@ -10572,7 +10572,7 @@
       <c r="H274" t="inlineStr"/>
       <c r="I274" t="inlineStr">
         <is>
-          <t>T2</t>
+          <t>DESC</t>
         </is>
       </c>
       <c r="J274" t="n">
@@ -11275,7 +11275,7 @@
       <c r="H293" t="inlineStr"/>
       <c r="I293" t="inlineStr">
         <is>
-          <t>T2</t>
+          <t>DESC</t>
         </is>
       </c>
       <c r="J293" t="n">
@@ -11312,11 +11312,11 @@
       <c r="H294" t="inlineStr"/>
       <c r="I294" t="inlineStr">
         <is>
-          <t>DESC</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="J294" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K294" t="n">
         <v>2</v>
@@ -11460,11 +11460,11 @@
       <c r="H298" t="inlineStr"/>
       <c r="I298" t="inlineStr">
         <is>
-          <t>T2</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="J298" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K298" t="n">
         <v>2</v>
@@ -11497,11 +11497,11 @@
       <c r="H299" t="inlineStr"/>
       <c r="I299" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J299" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K299" t="n">
         <v>2</v>
@@ -11571,7 +11571,7 @@
       <c r="H301" t="inlineStr"/>
       <c r="I301" t="inlineStr">
         <is>
-          <t>DESC</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="J301" t="n">
@@ -11608,11 +11608,11 @@
       <c r="H302" t="inlineStr"/>
       <c r="I302" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>DESC</t>
         </is>
       </c>
       <c r="J302" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K302" t="n">
         <v>2</v>
@@ -11645,11 +11645,11 @@
       <c r="H303" t="inlineStr"/>
       <c r="I303" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J303" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K303" t="n">
         <v>2</v>
@@ -11719,11 +11719,11 @@
       <c r="H305" t="inlineStr"/>
       <c r="I305" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="J305" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K305" t="n">
         <v>2</v>
@@ -11760,7 +11760,7 @@
         </is>
       </c>
       <c r="J306" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K306" t="n">
         <v>2</v>
@@ -11793,11 +11793,11 @@
       <c r="H307" t="inlineStr"/>
       <c r="I307" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J307" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K307" t="n">
         <v>2</v>
@@ -11867,11 +11867,11 @@
       <c r="H309" t="inlineStr"/>
       <c r="I309" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="J309" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K309" t="n">
         <v>2</v>
@@ -11908,7 +11908,7 @@
         </is>
       </c>
       <c r="J310" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K310" t="n">
         <v>2</v>
@@ -11941,11 +11941,11 @@
       <c r="H311" t="inlineStr"/>
       <c r="I311" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J311" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="K311" t="n">
         <v>2</v>
@@ -12015,11 +12015,11 @@
       <c r="H313" t="inlineStr"/>
       <c r="I313" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="J313" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K313" t="n">
         <v>2</v>
@@ -12056,7 +12056,7 @@
         </is>
       </c>
       <c r="J314" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K314" t="n">
         <v>2</v>
@@ -12089,11 +12089,11 @@
       <c r="H315" t="inlineStr"/>
       <c r="I315" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J315" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="K315" t="n">
         <v>2</v>
@@ -12163,11 +12163,11 @@
       <c r="H317" t="inlineStr"/>
       <c r="I317" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="J317" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="K317" t="n">
         <v>2</v>
@@ -12204,7 +12204,7 @@
         </is>
       </c>
       <c r="J318" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K318" t="n">
         <v>2</v>
@@ -12237,11 +12237,11 @@
       <c r="H319" t="inlineStr"/>
       <c r="I319" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J319" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="K319" t="n">
         <v>2</v>
@@ -12311,7 +12311,7 @@
       <c r="H321" t="inlineStr"/>
       <c r="I321" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>DESC</t>
         </is>
       </c>
       <c r="J321" t="n">
@@ -12348,11 +12348,11 @@
       <c r="H322" t="inlineStr"/>
       <c r="I322" t="inlineStr">
         <is>
-          <t>DESC</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="J322" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="K322" t="n">
         <v>2</v>
@@ -12459,11 +12459,11 @@
       <c r="H325" t="inlineStr"/>
       <c r="I325" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J325" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K325" t="n">
         <v>2</v>
@@ -12500,7 +12500,7 @@
         </is>
       </c>
       <c r="J326" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="K326" t="n">
         <v>2</v>
@@ -12607,7 +12607,7 @@
       <c r="H329" t="inlineStr"/>
       <c r="I329" t="inlineStr">
         <is>
-          <t>DESC</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="J329" t="n">
@@ -12644,11 +12644,11 @@
       <c r="H330" t="inlineStr"/>
       <c r="I330" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>DESC</t>
         </is>
       </c>
       <c r="J330" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K330" t="n">
         <v>2</v>
@@ -12681,7 +12681,7 @@
       <c r="H331" t="inlineStr"/>
       <c r="I331" t="inlineStr">
         <is>
-          <t>T2</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J331" t="n">
@@ -12755,7 +12755,7 @@
       <c r="H333" t="inlineStr"/>
       <c r="I333" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="J333" t="n">
@@ -12792,11 +12792,11 @@
       <c r="H334" t="inlineStr"/>
       <c r="I334" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J334" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K334" t="n">
         <v>2</v>
@@ -12903,7 +12903,7 @@
       <c r="H337" t="inlineStr"/>
       <c r="I337" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="J337" t="n">
@@ -12940,11 +12940,11 @@
       <c r="H338" t="inlineStr"/>
       <c r="I338" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J338" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="K338" t="n">
         <v>2</v>
@@ -13051,7 +13051,7 @@
       <c r="H341" t="inlineStr"/>
       <c r="I341" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="J341" t="n">
@@ -13088,11 +13088,11 @@
       <c r="H342" t="inlineStr"/>
       <c r="I342" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J342" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="K342" t="n">
         <v>2</v>
@@ -13199,7 +13199,7 @@
       <c r="H345" t="inlineStr"/>
       <c r="I345" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="J345" t="n">
@@ -13236,11 +13236,11 @@
       <c r="H346" t="inlineStr"/>
       <c r="I346" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J346" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="K346" t="n">
         <v>2</v>
@@ -13347,7 +13347,7 @@
       <c r="H349" t="inlineStr"/>
       <c r="I349" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>DESC</t>
         </is>
       </c>
       <c r="J349" t="n">
@@ -13384,7 +13384,7 @@
       <c r="H350" t="inlineStr"/>
       <c r="I350" t="inlineStr">
         <is>
-          <t>DESC</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="J350" t="n">
@@ -13532,11 +13532,11 @@
       <c r="H354" t="inlineStr"/>
       <c r="I354" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="J354" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K354" t="n">
         <v>2</v>
@@ -13643,7 +13643,7 @@
       <c r="H357" t="inlineStr"/>
       <c r="I357" t="inlineStr">
         <is>
-          <t>DESC</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J357" t="n">
@@ -13680,7 +13680,7 @@
       <c r="H358" t="inlineStr"/>
       <c r="I358" t="inlineStr">
         <is>
-          <t>T2</t>
+          <t>DESC</t>
         </is>
       </c>
       <c r="J358" t="n">
@@ -14383,7 +14383,7 @@
       <c r="H377" t="inlineStr"/>
       <c r="I377" t="inlineStr">
         <is>
-          <t>T2</t>
+          <t>DESC</t>
         </is>
       </c>
       <c r="J377" t="n">
@@ -14420,11 +14420,11 @@
       <c r="H378" t="inlineStr"/>
       <c r="I378" t="inlineStr">
         <is>
-          <t>DESC</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="J378" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K378" t="n">
         <v>2</v>
@@ -14568,11 +14568,11 @@
       <c r="H382" t="inlineStr"/>
       <c r="I382" t="inlineStr">
         <is>
-          <t>T2</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="J382" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K382" t="n">
         <v>2</v>
@@ -14605,11 +14605,11 @@
       <c r="H383" t="inlineStr"/>
       <c r="I383" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J383" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K383" t="n">
         <v>2</v>
@@ -14679,7 +14679,7 @@
       <c r="H385" t="inlineStr"/>
       <c r="I385" t="inlineStr">
         <is>
-          <t>DESC</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="J385" t="n">
@@ -14716,11 +14716,11 @@
       <c r="H386" t="inlineStr"/>
       <c r="I386" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>DESC</t>
         </is>
       </c>
       <c r="J386" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K386" t="n">
         <v>2</v>
@@ -14753,11 +14753,11 @@
       <c r="H387" t="inlineStr"/>
       <c r="I387" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J387" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K387" t="n">
         <v>2</v>
@@ -14827,11 +14827,11 @@
       <c r="H389" t="inlineStr"/>
       <c r="I389" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="J389" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K389" t="n">
         <v>2</v>
@@ -14868,7 +14868,7 @@
         </is>
       </c>
       <c r="J390" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K390" t="n">
         <v>2</v>
@@ -14901,11 +14901,11 @@
       <c r="H391" t="inlineStr"/>
       <c r="I391" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J391" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K391" t="n">
         <v>2</v>
@@ -14975,11 +14975,11 @@
       <c r="H393" t="inlineStr"/>
       <c r="I393" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="J393" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K393" t="n">
         <v>2</v>
@@ -15016,7 +15016,7 @@
         </is>
       </c>
       <c r="J394" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K394" t="n">
         <v>2</v>
@@ -15049,11 +15049,11 @@
       <c r="H395" t="inlineStr"/>
       <c r="I395" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J395" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="K395" t="n">
         <v>2</v>
@@ -15123,11 +15123,11 @@
       <c r="H397" t="inlineStr"/>
       <c r="I397" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="J397" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K397" t="n">
         <v>2</v>
@@ -15164,7 +15164,7 @@
         </is>
       </c>
       <c r="J398" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K398" t="n">
         <v>2</v>
@@ -15197,11 +15197,11 @@
       <c r="H399" t="inlineStr"/>
       <c r="I399" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J399" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="K399" t="n">
         <v>2</v>
@@ -15271,11 +15271,11 @@
       <c r="H401" t="inlineStr"/>
       <c r="I401" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="J401" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="K401" t="n">
         <v>2</v>
@@ -15312,7 +15312,7 @@
         </is>
       </c>
       <c r="J402" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K402" t="n">
         <v>2</v>
@@ -15345,11 +15345,11 @@
       <c r="H403" t="inlineStr"/>
       <c r="I403" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J403" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="K403" t="n">
         <v>2</v>
@@ -15419,7 +15419,7 @@
       <c r="H405" t="inlineStr"/>
       <c r="I405" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>DESC</t>
         </is>
       </c>
       <c r="J405" t="n">
@@ -15456,11 +15456,11 @@
       <c r="H406" t="inlineStr"/>
       <c r="I406" t="inlineStr">
         <is>
-          <t>DESC</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="J406" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="K406" t="n">
         <v>2</v>
@@ -15567,11 +15567,11 @@
       <c r="H409" t="inlineStr"/>
       <c r="I409" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J409" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K409" t="n">
         <v>2</v>
@@ -15608,7 +15608,7 @@
         </is>
       </c>
       <c r="J410" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="K410" t="n">
         <v>2</v>
@@ -15715,7 +15715,7 @@
       <c r="H413" t="inlineStr"/>
       <c r="I413" t="inlineStr">
         <is>
-          <t>DESC</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="J413" t="n">
@@ -15752,11 +15752,11 @@
       <c r="H414" t="inlineStr"/>
       <c r="I414" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>DESC</t>
         </is>
       </c>
       <c r="J414" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K414" t="n">
         <v>2</v>
@@ -15789,7 +15789,7 @@
       <c r="H415" t="inlineStr"/>
       <c r="I415" t="inlineStr">
         <is>
-          <t>T2</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J415" t="n">
@@ -15863,7 +15863,7 @@
       <c r="H417" t="inlineStr"/>
       <c r="I417" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="J417" t="n">
@@ -15900,11 +15900,11 @@
       <c r="H418" t="inlineStr"/>
       <c r="I418" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J418" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K418" t="n">
         <v>2</v>
@@ -16011,7 +16011,7 @@
       <c r="H421" t="inlineStr"/>
       <c r="I421" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="J421" t="n">
@@ -16048,11 +16048,11 @@
       <c r="H422" t="inlineStr"/>
       <c r="I422" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J422" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="K422" t="n">
         <v>2</v>
@@ -16159,7 +16159,7 @@
       <c r="H425" t="inlineStr"/>
       <c r="I425" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="J425" t="n">
@@ -16196,11 +16196,11 @@
       <c r="H426" t="inlineStr"/>
       <c r="I426" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J426" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="K426" t="n">
         <v>2</v>
@@ -16307,7 +16307,7 @@
       <c r="H429" t="inlineStr"/>
       <c r="I429" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="J429" t="n">
@@ -16344,11 +16344,11 @@
       <c r="H430" t="inlineStr"/>
       <c r="I430" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J430" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="K430" t="n">
         <v>2</v>
@@ -16455,7 +16455,7 @@
       <c r="H433" t="inlineStr"/>
       <c r="I433" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>DESC</t>
         </is>
       </c>
       <c r="J433" t="n">
@@ -16492,7 +16492,7 @@
       <c r="H434" t="inlineStr"/>
       <c r="I434" t="inlineStr">
         <is>
-          <t>DESC</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="J434" t="n">
@@ -16640,11 +16640,11 @@
       <c r="H438" t="inlineStr"/>
       <c r="I438" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="J438" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K438" t="n">
         <v>2</v>
@@ -16751,7 +16751,7 @@
       <c r="H441" t="inlineStr"/>
       <c r="I441" t="inlineStr">
         <is>
-          <t>DESC</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J441" t="n">
@@ -16788,7 +16788,7 @@
       <c r="H442" t="inlineStr"/>
       <c r="I442" t="inlineStr">
         <is>
-          <t>T2</t>
+          <t>DESC</t>
         </is>
       </c>
       <c r="J442" t="n">
@@ -17491,7 +17491,7 @@
       <c r="H461" t="inlineStr"/>
       <c r="I461" t="inlineStr">
         <is>
-          <t>T2</t>
+          <t>DESC</t>
         </is>
       </c>
       <c r="J461" t="n">
@@ -17528,11 +17528,11 @@
       <c r="H462" t="inlineStr"/>
       <c r="I462" t="inlineStr">
         <is>
-          <t>DESC</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="J462" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K462" t="n">
         <v>2</v>
@@ -17676,11 +17676,11 @@
       <c r="H466" t="inlineStr"/>
       <c r="I466" t="inlineStr">
         <is>
-          <t>T2</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="J466" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K466" t="n">
         <v>2</v>
@@ -17713,11 +17713,11 @@
       <c r="H467" t="inlineStr"/>
       <c r="I467" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J467" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K467" t="n">
         <v>2</v>
@@ -17787,7 +17787,7 @@
       <c r="H469" t="inlineStr"/>
       <c r="I469" t="inlineStr">
         <is>
-          <t>DESC</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="J469" t="n">
@@ -17824,11 +17824,11 @@
       <c r="H470" t="inlineStr"/>
       <c r="I470" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>DESC</t>
         </is>
       </c>
       <c r="J470" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K470" t="n">
         <v>2</v>
@@ -17861,11 +17861,11 @@
       <c r="H471" t="inlineStr"/>
       <c r="I471" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J471" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K471" t="n">
         <v>2</v>
@@ -17935,11 +17935,11 @@
       <c r="H473" t="inlineStr"/>
       <c r="I473" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="J473" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K473" t="n">
         <v>2</v>
@@ -17976,7 +17976,7 @@
         </is>
       </c>
       <c r="J474" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K474" t="n">
         <v>2</v>
@@ -18009,11 +18009,11 @@
       <c r="H475" t="inlineStr"/>
       <c r="I475" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J475" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K475" t="n">
         <v>2</v>
@@ -18083,11 +18083,11 @@
       <c r="H477" t="inlineStr"/>
       <c r="I477" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="J477" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K477" t="n">
         <v>2</v>
@@ -18124,7 +18124,7 @@
         </is>
       </c>
       <c r="J478" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K478" t="n">
         <v>2</v>
@@ -18157,11 +18157,11 @@
       <c r="H479" t="inlineStr"/>
       <c r="I479" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J479" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="K479" t="n">
         <v>2</v>
@@ -18231,11 +18231,11 @@
       <c r="H481" t="inlineStr"/>
       <c r="I481" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="J481" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K481" t="n">
         <v>2</v>
@@ -18272,7 +18272,7 @@
         </is>
       </c>
       <c r="J482" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K482" t="n">
         <v>2</v>
@@ -18305,11 +18305,11 @@
       <c r="H483" t="inlineStr"/>
       <c r="I483" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J483" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="K483" t="n">
         <v>2</v>
@@ -18379,11 +18379,11 @@
       <c r="H485" t="inlineStr"/>
       <c r="I485" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="J485" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="K485" t="n">
         <v>2</v>
@@ -18420,7 +18420,7 @@
         </is>
       </c>
       <c r="J486" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K486" t="n">
         <v>2</v>
@@ -18453,11 +18453,11 @@
       <c r="H487" t="inlineStr"/>
       <c r="I487" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J487" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="K487" t="n">
         <v>2</v>
@@ -18527,7 +18527,7 @@
       <c r="H489" t="inlineStr"/>
       <c r="I489" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>DESC</t>
         </is>
       </c>
       <c r="J489" t="n">
@@ -18564,11 +18564,11 @@
       <c r="H490" t="inlineStr"/>
       <c r="I490" t="inlineStr">
         <is>
-          <t>DESC</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="J490" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="K490" t="n">
         <v>2</v>
@@ -18675,11 +18675,11 @@
       <c r="H493" t="inlineStr"/>
       <c r="I493" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J493" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K493" t="n">
         <v>2</v>
@@ -18716,7 +18716,7 @@
         </is>
       </c>
       <c r="J494" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="K494" t="n">
         <v>2</v>
@@ -18823,7 +18823,7 @@
       <c r="H497" t="inlineStr"/>
       <c r="I497" t="inlineStr">
         <is>
-          <t>DESC</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="J497" t="n">
@@ -18860,11 +18860,11 @@
       <c r="H498" t="inlineStr"/>
       <c r="I498" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>DESC</t>
         </is>
       </c>
       <c r="J498" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K498" t="n">
         <v>2</v>
@@ -18897,7 +18897,7 @@
       <c r="H499" t="inlineStr"/>
       <c r="I499" t="inlineStr">
         <is>
-          <t>T2</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J499" t="n">
@@ -18971,7 +18971,7 @@
       <c r="H501" t="inlineStr"/>
       <c r="I501" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="J501" t="n">
@@ -19008,11 +19008,11 @@
       <c r="H502" t="inlineStr"/>
       <c r="I502" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J502" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K502" t="n">
         <v>2</v>
@@ -19119,7 +19119,7 @@
       <c r="H505" t="inlineStr"/>
       <c r="I505" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="J505" t="n">
@@ -19156,11 +19156,11 @@
       <c r="H506" t="inlineStr"/>
       <c r="I506" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J506" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="K506" t="n">
         <v>2</v>
@@ -19267,7 +19267,7 @@
       <c r="H509" t="inlineStr"/>
       <c r="I509" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="J509" t="n">
@@ -19304,11 +19304,11 @@
       <c r="H510" t="inlineStr"/>
       <c r="I510" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J510" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="K510" t="n">
         <v>2</v>
@@ -19415,7 +19415,7 @@
       <c r="H513" t="inlineStr"/>
       <c r="I513" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="J513" t="n">
@@ -19452,11 +19452,11 @@
       <c r="H514" t="inlineStr"/>
       <c r="I514" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J514" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="K514" t="n">
         <v>2</v>
@@ -19563,7 +19563,7 @@
       <c r="H517" t="inlineStr"/>
       <c r="I517" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>DESC</t>
         </is>
       </c>
       <c r="J517" t="n">
@@ -19600,7 +19600,7 @@
       <c r="H518" t="inlineStr"/>
       <c r="I518" t="inlineStr">
         <is>
-          <t>DESC</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="J518" t="n">
@@ -19748,11 +19748,11 @@
       <c r="H522" t="inlineStr"/>
       <c r="I522" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="J522" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K522" t="n">
         <v>2</v>
@@ -19859,7 +19859,7 @@
       <c r="H525" t="inlineStr"/>
       <c r="I525" t="inlineStr">
         <is>
-          <t>DESC</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J525" t="n">
@@ -19896,7 +19896,7 @@
       <c r="H526" t="inlineStr"/>
       <c r="I526" t="inlineStr">
         <is>
-          <t>T2</t>
+          <t>DESC</t>
         </is>
       </c>
       <c r="J526" t="n">
@@ -20599,7 +20599,7 @@
       <c r="H545" t="inlineStr"/>
       <c r="I545" t="inlineStr">
         <is>
-          <t>T2</t>
+          <t>DESC</t>
         </is>
       </c>
       <c r="J545" t="n">
@@ -20636,11 +20636,11 @@
       <c r="H546" t="inlineStr"/>
       <c r="I546" t="inlineStr">
         <is>
-          <t>DESC</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="J546" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K546" t="n">
         <v>2</v>
@@ -20784,11 +20784,11 @@
       <c r="H550" t="inlineStr"/>
       <c r="I550" t="inlineStr">
         <is>
-          <t>T2</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="J550" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K550" t="n">
         <v>2</v>
@@ -20821,11 +20821,11 @@
       <c r="H551" t="inlineStr"/>
       <c r="I551" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J551" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K551" t="n">
         <v>2</v>
@@ -20895,7 +20895,7 @@
       <c r="H553" t="inlineStr"/>
       <c r="I553" t="inlineStr">
         <is>
-          <t>DESC</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="J553" t="n">
@@ -20932,11 +20932,11 @@
       <c r="H554" t="inlineStr"/>
       <c r="I554" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>DESC</t>
         </is>
       </c>
       <c r="J554" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K554" t="n">
         <v>2</v>
@@ -20969,11 +20969,11 @@
       <c r="H555" t="inlineStr"/>
       <c r="I555" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J555" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K555" t="n">
         <v>2</v>
@@ -21043,11 +21043,11 @@
       <c r="H557" t="inlineStr"/>
       <c r="I557" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="J557" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K557" t="n">
         <v>2</v>
@@ -21084,7 +21084,7 @@
         </is>
       </c>
       <c r="J558" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K558" t="n">
         <v>2</v>
@@ -21117,11 +21117,11 @@
       <c r="H559" t="inlineStr"/>
       <c r="I559" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J559" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K559" t="n">
         <v>2</v>
@@ -21191,11 +21191,11 @@
       <c r="H561" t="inlineStr"/>
       <c r="I561" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="J561" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K561" t="n">
         <v>2</v>
@@ -21232,7 +21232,7 @@
         </is>
       </c>
       <c r="J562" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K562" t="n">
         <v>2</v>
@@ -21265,11 +21265,11 @@
       <c r="H563" t="inlineStr"/>
       <c r="I563" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J563" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="K563" t="n">
         <v>2</v>
@@ -21339,11 +21339,11 @@
       <c r="H565" t="inlineStr"/>
       <c r="I565" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="J565" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K565" t="n">
         <v>2</v>
@@ -21380,7 +21380,7 @@
         </is>
       </c>
       <c r="J566" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K566" t="n">
         <v>2</v>
@@ -21413,11 +21413,11 @@
       <c r="H567" t="inlineStr"/>
       <c r="I567" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J567" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="K567" t="n">
         <v>2</v>
@@ -21487,11 +21487,11 @@
       <c r="H569" t="inlineStr"/>
       <c r="I569" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="J569" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="K569" t="n">
         <v>2</v>
@@ -21528,7 +21528,7 @@
         </is>
       </c>
       <c r="J570" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K570" t="n">
         <v>2</v>
@@ -21561,11 +21561,11 @@
       <c r="H571" t="inlineStr"/>
       <c r="I571" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J571" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="K571" t="n">
         <v>2</v>
@@ -21635,7 +21635,7 @@
       <c r="H573" t="inlineStr"/>
       <c r="I573" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>DESC</t>
         </is>
       </c>
       <c r="J573" t="n">
@@ -21672,11 +21672,11 @@
       <c r="H574" t="inlineStr"/>
       <c r="I574" t="inlineStr">
         <is>
-          <t>DESC</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="J574" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="K574" t="n">
         <v>2</v>
@@ -21783,11 +21783,11 @@
       <c r="H577" t="inlineStr"/>
       <c r="I577" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J577" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K577" t="n">
         <v>2</v>
@@ -21824,7 +21824,7 @@
         </is>
       </c>
       <c r="J578" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="K578" t="n">
         <v>2</v>
@@ -21931,7 +21931,7 @@
       <c r="H581" t="inlineStr"/>
       <c r="I581" t="inlineStr">
         <is>
-          <t>DESC</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="J581" t="n">
@@ -21968,11 +21968,11 @@
       <c r="H582" t="inlineStr"/>
       <c r="I582" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>DESC</t>
         </is>
       </c>
       <c r="J582" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K582" t="n">
         <v>2</v>
@@ -22005,7 +22005,7 @@
       <c r="H583" t="inlineStr"/>
       <c r="I583" t="inlineStr">
         <is>
-          <t>T2</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J583" t="n">
@@ -22079,7 +22079,7 @@
       <c r="H585" t="inlineStr"/>
       <c r="I585" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="J585" t="n">
@@ -22116,11 +22116,11 @@
       <c r="H586" t="inlineStr"/>
       <c r="I586" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J586" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K586" t="n">
         <v>2</v>
@@ -22227,7 +22227,7 @@
       <c r="H589" t="inlineStr"/>
       <c r="I589" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="J589" t="n">
@@ -22264,11 +22264,11 @@
       <c r="H590" t="inlineStr"/>
       <c r="I590" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J590" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="K590" t="n">
         <v>2</v>
@@ -22375,7 +22375,7 @@
       <c r="H593" t="inlineStr"/>
       <c r="I593" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="J593" t="n">
@@ -22412,11 +22412,11 @@
       <c r="H594" t="inlineStr"/>
       <c r="I594" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J594" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="K594" t="n">
         <v>2</v>
@@ -22523,7 +22523,7 @@
       <c r="H597" t="inlineStr"/>
       <c r="I597" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="J597" t="n">
@@ -22560,11 +22560,11 @@
       <c r="H598" t="inlineStr"/>
       <c r="I598" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J598" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="K598" t="n">
         <v>2</v>
@@ -22671,7 +22671,7 @@
       <c r="H601" t="inlineStr"/>
       <c r="I601" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>DESC</t>
         </is>
       </c>
       <c r="J601" t="n">
@@ -22708,7 +22708,7 @@
       <c r="H602" t="inlineStr"/>
       <c r="I602" t="inlineStr">
         <is>
-          <t>DESC</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="J602" t="n">
@@ -22856,11 +22856,11 @@
       <c r="H606" t="inlineStr"/>
       <c r="I606" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="J606" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K606" t="n">
         <v>2</v>
@@ -22967,7 +22967,7 @@
       <c r="H609" t="inlineStr"/>
       <c r="I609" t="inlineStr">
         <is>
-          <t>DESC</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J609" t="n">
@@ -23004,7 +23004,7 @@
       <c r="H610" t="inlineStr"/>
       <c r="I610" t="inlineStr">
         <is>
-          <t>T2</t>
+          <t>DESC</t>
         </is>
       </c>
       <c r="J610" t="n">
@@ -23707,7 +23707,7 @@
       <c r="H629" t="inlineStr"/>
       <c r="I629" t="inlineStr">
         <is>
-          <t>T2</t>
+          <t>DESC</t>
         </is>
       </c>
       <c r="J629" t="n">
@@ -23744,11 +23744,11 @@
       <c r="H630" t="inlineStr"/>
       <c r="I630" t="inlineStr">
         <is>
-          <t>DESC</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="J630" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K630" t="n">
         <v>2</v>
@@ -23892,11 +23892,11 @@
       <c r="H634" t="inlineStr"/>
       <c r="I634" t="inlineStr">
         <is>
-          <t>T2</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="J634" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K634" t="n">
         <v>2</v>
@@ -23929,11 +23929,11 @@
       <c r="H635" t="inlineStr"/>
       <c r="I635" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J635" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K635" t="n">
         <v>2</v>
@@ -24003,7 +24003,7 @@
       <c r="H637" t="inlineStr"/>
       <c r="I637" t="inlineStr">
         <is>
-          <t>DESC</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="J637" t="n">
@@ -24040,11 +24040,11 @@
       <c r="H638" t="inlineStr"/>
       <c r="I638" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>DESC</t>
         </is>
       </c>
       <c r="J638" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K638" t="n">
         <v>2</v>
@@ -24077,11 +24077,11 @@
       <c r="H639" t="inlineStr"/>
       <c r="I639" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J639" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K639" t="n">
         <v>2</v>
@@ -24151,11 +24151,11 @@
       <c r="H641" t="inlineStr"/>
       <c r="I641" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="J641" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K641" t="n">
         <v>2</v>
@@ -24192,7 +24192,7 @@
         </is>
       </c>
       <c r="J642" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K642" t="n">
         <v>2</v>
@@ -24225,11 +24225,11 @@
       <c r="H643" t="inlineStr"/>
       <c r="I643" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J643" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K643" t="n">
         <v>2</v>
@@ -24299,11 +24299,11 @@
       <c r="H645" t="inlineStr"/>
       <c r="I645" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="J645" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K645" t="n">
         <v>2</v>
@@ -24340,7 +24340,7 @@
         </is>
       </c>
       <c r="J646" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K646" t="n">
         <v>2</v>
@@ -24373,11 +24373,11 @@
       <c r="H647" t="inlineStr"/>
       <c r="I647" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J647" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="K647" t="n">
         <v>2</v>
@@ -24447,11 +24447,11 @@
       <c r="H649" t="inlineStr"/>
       <c r="I649" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="J649" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K649" t="n">
         <v>2</v>
@@ -24488,7 +24488,7 @@
         </is>
       </c>
       <c r="J650" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K650" t="n">
         <v>2</v>
@@ -24521,11 +24521,11 @@
       <c r="H651" t="inlineStr"/>
       <c r="I651" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J651" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="K651" t="n">
         <v>2</v>
@@ -24595,11 +24595,11 @@
       <c r="H653" t="inlineStr"/>
       <c r="I653" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="J653" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="K653" t="n">
         <v>2</v>
@@ -24636,7 +24636,7 @@
         </is>
       </c>
       <c r="J654" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K654" t="n">
         <v>2</v>
@@ -24669,11 +24669,11 @@
       <c r="H655" t="inlineStr"/>
       <c r="I655" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J655" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="K655" t="n">
         <v>2</v>
@@ -24743,7 +24743,7 @@
       <c r="H657" t="inlineStr"/>
       <c r="I657" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>DESC</t>
         </is>
       </c>
       <c r="J657" t="n">
@@ -24780,11 +24780,11 @@
       <c r="H658" t="inlineStr"/>
       <c r="I658" t="inlineStr">
         <is>
-          <t>DESC</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="J658" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="K658" t="n">
         <v>2</v>
@@ -24891,11 +24891,11 @@
       <c r="H661" t="inlineStr"/>
       <c r="I661" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J661" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K661" t="n">
         <v>2</v>
@@ -24932,7 +24932,7 @@
         </is>
       </c>
       <c r="J662" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="K662" t="n">
         <v>2</v>
@@ -25039,7 +25039,7 @@
       <c r="H665" t="inlineStr"/>
       <c r="I665" t="inlineStr">
         <is>
-          <t>DESC</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="J665" t="n">
@@ -25076,11 +25076,11 @@
       <c r="H666" t="inlineStr"/>
       <c r="I666" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>DESC</t>
         </is>
       </c>
       <c r="J666" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K666" t="n">
         <v>2</v>
@@ -25113,7 +25113,7 @@
       <c r="H667" t="inlineStr"/>
       <c r="I667" t="inlineStr">
         <is>
-          <t>T2</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J667" t="n">
@@ -25187,7 +25187,7 @@
       <c r="H669" t="inlineStr"/>
       <c r="I669" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="J669" t="n">
@@ -25224,11 +25224,11 @@
       <c r="H670" t="inlineStr"/>
       <c r="I670" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J670" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K670" t="n">
         <v>2</v>
@@ -25335,7 +25335,7 @@
       <c r="H673" t="inlineStr"/>
       <c r="I673" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="J673" t="n">
@@ -25372,11 +25372,11 @@
       <c r="H674" t="inlineStr"/>
       <c r="I674" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J674" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="K674" t="n">
         <v>2</v>
@@ -25483,7 +25483,7 @@
       <c r="H677" t="inlineStr"/>
       <c r="I677" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="J677" t="n">
@@ -25520,11 +25520,11 @@
       <c r="H678" t="inlineStr"/>
       <c r="I678" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J678" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="K678" t="n">
         <v>2</v>
@@ -25631,7 +25631,7 @@
       <c r="H681" t="inlineStr"/>
       <c r="I681" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="J681" t="n">
@@ -25668,11 +25668,11 @@
       <c r="H682" t="inlineStr"/>
       <c r="I682" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J682" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="K682" t="n">
         <v>2</v>
@@ -25779,7 +25779,7 @@
       <c r="H685" t="inlineStr"/>
       <c r="I685" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>DESC</t>
         </is>
       </c>
       <c r="J685" t="n">
@@ -25816,7 +25816,7 @@
       <c r="H686" t="inlineStr"/>
       <c r="I686" t="inlineStr">
         <is>
-          <t>DESC</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="J686" t="n">
@@ -25964,11 +25964,11 @@
       <c r="H690" t="inlineStr"/>
       <c r="I690" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="J690" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K690" t="n">
         <v>2</v>
@@ -26075,7 +26075,7 @@
       <c r="H693" t="inlineStr"/>
       <c r="I693" t="inlineStr">
         <is>
-          <t>DESC</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J693" t="n">
@@ -26112,7 +26112,7 @@
       <c r="H694" t="inlineStr"/>
       <c r="I694" t="inlineStr">
         <is>
-          <t>T2</t>
+          <t>DESC</t>
         </is>
       </c>
       <c r="J694" t="n">
@@ -26815,7 +26815,7 @@
       <c r="H713" t="inlineStr"/>
       <c r="I713" t="inlineStr">
         <is>
-          <t>T2</t>
+          <t>DESC</t>
         </is>
       </c>
       <c r="J713" t="n">
@@ -26852,11 +26852,11 @@
       <c r="H714" t="inlineStr"/>
       <c r="I714" t="inlineStr">
         <is>
-          <t>DESC</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="J714" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K714" t="n">
         <v>2</v>
@@ -27000,11 +27000,11 @@
       <c r="H718" t="inlineStr"/>
       <c r="I718" t="inlineStr">
         <is>
-          <t>T2</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="J718" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K718" t="n">
         <v>2</v>
@@ -27037,11 +27037,11 @@
       <c r="H719" t="inlineStr"/>
       <c r="I719" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J719" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K719" t="n">
         <v>2</v>
@@ -27111,7 +27111,7 @@
       <c r="H721" t="inlineStr"/>
       <c r="I721" t="inlineStr">
         <is>
-          <t>DESC</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="J721" t="n">
@@ -27148,11 +27148,11 @@
       <c r="H722" t="inlineStr"/>
       <c r="I722" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>DESC</t>
         </is>
       </c>
       <c r="J722" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K722" t="n">
         <v>2</v>
@@ -27185,11 +27185,11 @@
       <c r="H723" t="inlineStr"/>
       <c r="I723" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J723" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K723" t="n">
         <v>2</v>
@@ -27259,11 +27259,11 @@
       <c r="H725" t="inlineStr"/>
       <c r="I725" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="J725" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K725" t="n">
         <v>2</v>
@@ -27300,7 +27300,7 @@
         </is>
       </c>
       <c r="J726" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K726" t="n">
         <v>2</v>
@@ -27333,11 +27333,11 @@
       <c r="H727" t="inlineStr"/>
       <c r="I727" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J727" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K727" t="n">
         <v>2</v>
@@ -27407,11 +27407,11 @@
       <c r="H729" t="inlineStr"/>
       <c r="I729" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="J729" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K729" t="n">
         <v>2</v>
@@ -27448,7 +27448,7 @@
         </is>
       </c>
       <c r="J730" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K730" t="n">
         <v>2</v>
@@ -27481,11 +27481,11 @@
       <c r="H731" t="inlineStr"/>
       <c r="I731" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J731" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="K731" t="n">
         <v>2</v>
@@ -27555,11 +27555,11 @@
       <c r="H733" t="inlineStr"/>
       <c r="I733" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="J733" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K733" t="n">
         <v>2</v>
@@ -27596,7 +27596,7 @@
         </is>
       </c>
       <c r="J734" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K734" t="n">
         <v>2</v>
@@ -27629,11 +27629,11 @@
       <c r="H735" t="inlineStr"/>
       <c r="I735" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="J735" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="K735" t="n">
         <v>2</v>
@@ -27703,11 +27703,11 @@
       <c r="H737" t="inlineStr"/>
       <c r="I737" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="J737" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="K737" t="n">
         <v>2</v>

</xml_diff>